<commit_message>
Working on the correctness of the model.
</commit_message>
<xml_diff>
--- a/Projects/ARK_RWS/images/peilbuizen/pb_tauw_XY.xlsx
+++ b/Projects/ARK_RWS/images/peilbuizen/pb_tauw_XY.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Theo/Development/python/mf6_tools/mf6lab/Projects/ARK_RWS/images/peilbuizen/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90EF5F07-E3D4-154B-B24F-5834BC2E0EF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53DB8952-83CA-9D46-9650-2652E78A518A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8160" yWindow="11880" windowWidth="25340" windowHeight="20720" activeTab="4" xr2:uid="{E4383F88-647D-C347-BE79-FF24D0CA7E92}"/>
+    <workbookView xWindow="8160" yWindow="1680" windowWidth="25340" windowHeight="20720" activeTab="5" xr2:uid="{E4383F88-647D-C347-BE79-FF24D0CA7E92}"/>
   </bookViews>
   <sheets>
     <sheet name="pbTauw" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,8 @@
     <sheet name="joined" sheetId="5" r:id="rId3"/>
     <sheet name="Sheet2" sheetId="4" r:id="rId4"/>
     <sheet name="laagopbouw" sheetId="6" r:id="rId5"/>
+    <sheet name="wellen" sheetId="7" r:id="rId6"/>
+    <sheet name="raaien" sheetId="8" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="yyy" comment="Tijden en waarden van de stijghoogten gemiddeld over ca. 1 maand">Sheet2!$A$1:$G$67</definedName>
@@ -198,7 +200,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="119">
   <si>
     <t>x</t>
   </si>
@@ -544,6 +546,18 @@
   <si>
     <t>kD</t>
   </si>
+  <si>
+    <t>ymean</t>
+  </si>
+  <si>
+    <t>ymax</t>
+  </si>
+  <si>
+    <t>ymin</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
 </sst>
 </file>
 
@@ -552,7 +566,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -561,9 +575,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -587,13 +608,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1063,13 +1089,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9242C9A1-0ECC-C140-AC02-EB1C99BC61A4}">
-  <dimension ref="A1:N78"/>
+  <dimension ref="A1:P78"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="12" max="14" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1112,8 +1138,14 @@
       <c r="N1" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O1" t="s">
+        <v>89</v>
+      </c>
+      <c r="P1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>101</v>
       </c>
@@ -1153,15 +1185,21 @@
         <v>0</v>
       </c>
       <c r="M2">
-        <f t="shared" ref="M2:M33" si="1">VLOOKUP("Pb"&amp;$A2,yyy,6,FALSE)</f>
+        <f t="shared" ref="M2:O33" si="1">VLOOKUP("Pb"&amp;$A2,yyy,6,FALSE)</f>
         <v>-1.6919999999999999</v>
       </c>
       <c r="N2">
-        <f t="shared" ref="N2:N33" si="2">VLOOKUP("Pb"&amp;$A2,yyy,7,FALSE)</f>
+        <f t="shared" ref="N2:P33" si="2">VLOOKUP("Pb"&amp;$A2,yyy,7,FALSE)</f>
         <v>-1.78</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O2">
+        <v>-1.6919999999999999</v>
+      </c>
+      <c r="P2">
+        <v>-1.78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>102</v>
       </c>
@@ -1208,8 +1246,14 @@
         <f t="shared" si="2"/>
         <v>-1.841</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O3">
+        <v>-1.7390000000000001</v>
+      </c>
+      <c r="P3">
+        <v>-1.841</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>201</v>
       </c>
@@ -1256,8 +1300,14 @@
         <f t="shared" si="2"/>
         <v>-1.6839999999999999</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O4">
+        <v>-1.4810000000000001</v>
+      </c>
+      <c r="P4">
+        <v>-1.6839999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>202</v>
       </c>
@@ -1304,8 +1354,14 @@
         <f t="shared" si="2"/>
         <v>-1.7</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O5">
+        <v>-1.49</v>
+      </c>
+      <c r="P5">
+        <v>-1.7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>301</v>
       </c>
@@ -1352,8 +1408,14 @@
         <f t="shared" si="2"/>
         <v>-1.6539999999999999</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6">
+        <v>-1.6539999999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>302</v>
       </c>
@@ -1400,8 +1462,14 @@
         <f t="shared" si="2"/>
         <v>-1.556</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O7">
+        <v>-1.2350000000000001</v>
+      </c>
+      <c r="P7">
+        <v>-1.556</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>303</v>
       </c>
@@ -1448,8 +1516,14 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O8">
+        <v>-1.1160000000000001</v>
+      </c>
+      <c r="P8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>304</v>
       </c>
@@ -1496,8 +1570,14 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O9">
+        <v>-1.262</v>
+      </c>
+      <c r="P9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9002</v>
       </c>
@@ -1532,20 +1612,23 @@
         <f t="shared" si="3"/>
         <v>W</v>
       </c>
-      <c r="L10" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M10" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N10" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
+      <c r="P10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>401</v>
       </c>
@@ -1592,8 +1675,14 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O11">
+        <v>0</v>
+      </c>
+      <c r="P11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>402</v>
       </c>
@@ -1628,20 +1717,23 @@
         <f t="shared" si="3"/>
         <v>W</v>
       </c>
-      <c r="L12" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M12" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N12" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>0</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+      <c r="O12">
+        <v>0</v>
+      </c>
+      <c r="P12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>403</v>
       </c>
@@ -1676,20 +1768,23 @@
         <f t="shared" si="3"/>
         <v>W</v>
       </c>
-      <c r="L13" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M13" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N13" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L13">
+        <v>0</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13">
+        <v>0</v>
+      </c>
+      <c r="O13">
+        <v>0</v>
+      </c>
+      <c r="P13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>404</v>
       </c>
@@ -1724,20 +1819,23 @@
         <f t="shared" si="3"/>
         <v>W</v>
       </c>
-      <c r="L14" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M14" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N14" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+      <c r="N14">
+        <v>0</v>
+      </c>
+      <c r="O14">
+        <v>0</v>
+      </c>
+      <c r="P14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>405</v>
       </c>
@@ -1772,20 +1870,23 @@
         <f t="shared" si="3"/>
         <v>W</v>
       </c>
-      <c r="L15" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M15" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N15" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L15">
+        <v>0</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
+      </c>
+      <c r="N15">
+        <v>0</v>
+      </c>
+      <c r="O15">
+        <v>0</v>
+      </c>
+      <c r="P15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>406</v>
       </c>
@@ -1832,8 +1933,14 @@
         <f t="shared" si="2"/>
         <v>-1.49</v>
       </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O16">
+        <v>-0.998</v>
+      </c>
+      <c r="P16">
+        <v>-1.49</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>407</v>
       </c>
@@ -1880,8 +1987,14 @@
         <f t="shared" si="2"/>
         <v>-1.542</v>
       </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O17">
+        <v>-1.1040000000000001</v>
+      </c>
+      <c r="P17">
+        <v>-1.542</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>408</v>
       </c>
@@ -1916,20 +2029,23 @@
         <f t="shared" si="3"/>
         <v>E</v>
       </c>
-      <c r="L18" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M18" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N18" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L18">
+        <v>0</v>
+      </c>
+      <c r="M18">
+        <v>0</v>
+      </c>
+      <c r="N18">
+        <v>0</v>
+      </c>
+      <c r="O18">
+        <v>0</v>
+      </c>
+      <c r="P18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>409</v>
       </c>
@@ -1964,20 +2080,23 @@
         <f t="shared" si="3"/>
         <v>E</v>
       </c>
-      <c r="L19" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M19" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N19" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L19">
+        <v>0</v>
+      </c>
+      <c r="M19">
+        <v>0</v>
+      </c>
+      <c r="N19">
+        <v>0</v>
+      </c>
+      <c r="O19">
+        <v>0</v>
+      </c>
+      <c r="P19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>410</v>
       </c>
@@ -2024,8 +2143,14 @@
         <f t="shared" si="2"/>
         <v>-1.6220000000000001</v>
       </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O20">
+        <v>-1.399</v>
+      </c>
+      <c r="P20">
+        <v>-1.6220000000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>411</v>
       </c>
@@ -2072,8 +2197,14 @@
         <f t="shared" si="2"/>
         <v>-1.66</v>
       </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O21">
+        <v>-1.4470000000000001</v>
+      </c>
+      <c r="P21">
+        <v>-1.66</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>412</v>
       </c>
@@ -2120,8 +2251,14 @@
         <f t="shared" si="2"/>
         <v>-1.669</v>
       </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O22">
+        <v>-1.472</v>
+      </c>
+      <c r="P22">
+        <v>-1.669</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>501</v>
       </c>
@@ -2156,20 +2293,23 @@
         <f t="shared" si="3"/>
         <v>W</v>
       </c>
-      <c r="L23" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M23" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N23" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L23">
+        <v>0</v>
+      </c>
+      <c r="M23">
+        <v>0</v>
+      </c>
+      <c r="N23">
+        <v>0</v>
+      </c>
+      <c r="O23">
+        <v>0</v>
+      </c>
+      <c r="P23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>502</v>
       </c>
@@ -2204,20 +2344,23 @@
         <f t="shared" si="3"/>
         <v>W</v>
       </c>
-      <c r="L24" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M24" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N24" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L24">
+        <v>0</v>
+      </c>
+      <c r="M24">
+        <v>0</v>
+      </c>
+      <c r="N24">
+        <v>0</v>
+      </c>
+      <c r="O24">
+        <v>0</v>
+      </c>
+      <c r="P24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>503</v>
       </c>
@@ -2264,8 +2407,14 @@
         <f t="shared" si="2"/>
         <v>-1.734</v>
       </c>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O25">
+        <v>-1.542</v>
+      </c>
+      <c r="P25">
+        <v>-1.734</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>504</v>
       </c>
@@ -2312,8 +2461,14 @@
         <f t="shared" si="2"/>
         <v>-1.5529999999999999</v>
       </c>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O26">
+        <v>0</v>
+      </c>
+      <c r="P26">
+        <v>-1.5529999999999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>505</v>
       </c>
@@ -2360,8 +2515,14 @@
         <f t="shared" si="2"/>
         <v>-1.6220000000000001</v>
       </c>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O27">
+        <v>-1.2849999999999999</v>
+      </c>
+      <c r="P27">
+        <v>-1.6220000000000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>506</v>
       </c>
@@ -2408,8 +2569,14 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O28">
+        <v>-1.0680000000000001</v>
+      </c>
+      <c r="P28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>507</v>
       </c>
@@ -2444,20 +2611,23 @@
         <f t="shared" si="3"/>
         <v>E</v>
       </c>
-      <c r="L29" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M29" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N29" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L29">
+        <v>0</v>
+      </c>
+      <c r="M29">
+        <v>0</v>
+      </c>
+      <c r="N29">
+        <v>0</v>
+      </c>
+      <c r="O29">
+        <v>0</v>
+      </c>
+      <c r="P29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>508</v>
       </c>
@@ -2504,8 +2674,14 @@
         <f t="shared" si="2"/>
         <v>-1.821</v>
       </c>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O30">
+        <v>-1.538</v>
+      </c>
+      <c r="P30">
+        <v>-1.821</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>509</v>
       </c>
@@ -2552,8 +2728,14 @@
         <f t="shared" si="2"/>
         <v>-1.8080000000000001</v>
       </c>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O31">
+        <v>0</v>
+      </c>
+      <c r="P31">
+        <v>-1.8080000000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>510</v>
       </c>
@@ -2600,8 +2782,14 @@
         <f t="shared" si="2"/>
         <v>-1.7</v>
       </c>
-    </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O32">
+        <v>-1.5189999999999999</v>
+      </c>
+      <c r="P32">
+        <v>-1.7</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>511</v>
       </c>
@@ -2648,8 +2836,14 @@
         <f t="shared" si="2"/>
         <v>-1.698</v>
       </c>
-    </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O33">
+        <v>-1.506</v>
+      </c>
+      <c r="P33">
+        <v>-1.698</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>512</v>
       </c>
@@ -2684,20 +2878,23 @@
         <f t="shared" si="3"/>
         <v>E</v>
       </c>
-      <c r="L34" t="e">
-        <f t="shared" ref="L34:L65" si="6">VLOOKUP("Pb"&amp;$A34,yyy,5,FALSE)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="M34" t="e">
-        <f t="shared" ref="M34:M65" si="7">VLOOKUP("Pb"&amp;$A34,yyy,6,FALSE)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="N34" t="e">
-        <f t="shared" ref="N34:N65" si="8">VLOOKUP("Pb"&amp;$A34,yyy,7,FALSE)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L34">
+        <v>0</v>
+      </c>
+      <c r="M34">
+        <v>0</v>
+      </c>
+      <c r="N34">
+        <v>0</v>
+      </c>
+      <c r="O34">
+        <v>0</v>
+      </c>
+      <c r="P34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>601</v>
       </c>
@@ -2733,19 +2930,25 @@
         <v>W</v>
       </c>
       <c r="L35">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="L34:L65" si="6">VLOOKUP("Pb"&amp;$A35,yyy,5,FALSE)</f>
         <v>0</v>
       </c>
       <c r="M35">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="M34:O65" si="7">VLOOKUP("Pb"&amp;$A35,yyy,6,FALSE)</f>
         <v>-1.5580000000000001</v>
       </c>
       <c r="N35">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="N34:P65" si="8">VLOOKUP("Pb"&amp;$A35,yyy,7,FALSE)</f>
         <v>-1.698</v>
       </c>
-    </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O35">
+        <v>-1.5580000000000001</v>
+      </c>
+      <c r="P35">
+        <v>-1.698</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>602</v>
       </c>
@@ -2792,8 +2995,14 @@
         <f t="shared" si="8"/>
         <v>-1.6359999999999999</v>
       </c>
-    </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O36">
+        <v>-1.415</v>
+      </c>
+      <c r="P36">
+        <v>-1.6359999999999999</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>603</v>
       </c>
@@ -2840,8 +3049,14 @@
         <f t="shared" si="8"/>
         <v>-1.4850000000000001</v>
       </c>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O37">
+        <v>-1.196</v>
+      </c>
+      <c r="P37">
+        <v>-1.4850000000000001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>604</v>
       </c>
@@ -2876,20 +3091,23 @@
         <f t="shared" si="3"/>
         <v>E</v>
       </c>
-      <c r="L38" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M38" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N38" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L38">
+        <v>0</v>
+      </c>
+      <c r="M38">
+        <v>0</v>
+      </c>
+      <c r="N38">
+        <v>0</v>
+      </c>
+      <c r="O38">
+        <v>0</v>
+      </c>
+      <c r="P38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>605</v>
       </c>
@@ -2936,8 +3154,14 @@
         <f t="shared" si="8"/>
         <v>-1.6</v>
       </c>
-    </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O39">
+        <v>-1.3740000000000001</v>
+      </c>
+      <c r="P39">
+        <v>-1.6</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>606</v>
       </c>
@@ -2984,8 +3208,14 @@
         <f t="shared" si="8"/>
         <v>-1.6060000000000001</v>
       </c>
-    </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O40">
+        <v>0</v>
+      </c>
+      <c r="P40">
+        <v>-1.6060000000000001</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>701</v>
       </c>
@@ -3032,8 +3262,14 @@
         <f t="shared" si="8"/>
         <v>-1.7130000000000001</v>
       </c>
-    </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O41">
+        <v>-1.6120000000000001</v>
+      </c>
+      <c r="P41">
+        <v>-1.7130000000000001</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>702</v>
       </c>
@@ -3080,8 +3316,14 @@
         <f t="shared" si="8"/>
         <v>-1.4239999999999999</v>
       </c>
-    </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O42">
+        <v>-1.036</v>
+      </c>
+      <c r="P42">
+        <v>-1.4239999999999999</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>703</v>
       </c>
@@ -3128,8 +3370,14 @@
         <f t="shared" si="8"/>
         <v>-1.3939999999999999</v>
       </c>
-    </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O43">
+        <v>0</v>
+      </c>
+      <c r="P43">
+        <v>-1.3939999999999999</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>704</v>
       </c>
@@ -3164,20 +3412,23 @@
         <f t="shared" si="3"/>
         <v>E</v>
       </c>
-      <c r="L44" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M44" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N44" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L44">
+        <v>0</v>
+      </c>
+      <c r="M44">
+        <v>0</v>
+      </c>
+      <c r="N44">
+        <v>0</v>
+      </c>
+      <c r="O44">
+        <v>0</v>
+      </c>
+      <c r="P44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>801</v>
       </c>
@@ -3224,8 +3475,14 @@
         <f t="shared" si="8"/>
         <v>-2.6360000000000001</v>
       </c>
-    </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O45">
+        <v>-2.472</v>
+      </c>
+      <c r="P45">
+        <v>-2.6360000000000001</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>802</v>
       </c>
@@ -3272,8 +3529,14 @@
         <f t="shared" si="8"/>
         <v>-1.524</v>
       </c>
-    </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O46">
+        <v>-1.341</v>
+      </c>
+      <c r="P46">
+        <v>-1.524</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>803</v>
       </c>
@@ -3308,20 +3571,23 @@
         <f t="shared" si="3"/>
         <v>E</v>
       </c>
-      <c r="L47" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M47" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N47" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L47">
+        <v>0</v>
+      </c>
+      <c r="M47">
+        <v>0</v>
+      </c>
+      <c r="N47">
+        <v>0</v>
+      </c>
+      <c r="O47">
+        <v>0</v>
+      </c>
+      <c r="P47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>804</v>
       </c>
@@ -3356,20 +3622,23 @@
         <f t="shared" si="3"/>
         <v>E</v>
       </c>
-      <c r="L48" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M48" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N48" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L48">
+        <v>0</v>
+      </c>
+      <c r="M48">
+        <v>0</v>
+      </c>
+      <c r="N48">
+        <v>0</v>
+      </c>
+      <c r="O48">
+        <v>0</v>
+      </c>
+      <c r="P48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>805</v>
       </c>
@@ -3404,20 +3673,23 @@
         <f t="shared" si="3"/>
         <v>E</v>
       </c>
-      <c r="L49" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M49" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N49" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L49">
+        <v>0</v>
+      </c>
+      <c r="M49">
+        <v>0</v>
+      </c>
+      <c r="N49">
+        <v>0</v>
+      </c>
+      <c r="O49">
+        <v>0</v>
+      </c>
+      <c r="P49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>901</v>
       </c>
@@ -3464,8 +3736,14 @@
         <f t="shared" si="8"/>
         <v>-1.5209999999999999</v>
       </c>
-    </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O50">
+        <v>0</v>
+      </c>
+      <c r="P50">
+        <v>-1.5209999999999999</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>902</v>
       </c>
@@ -3512,8 +3790,14 @@
         <f t="shared" si="8"/>
         <v>-1.5509999999999999</v>
       </c>
-    </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O51">
+        <v>-1.395</v>
+      </c>
+      <c r="P51">
+        <v>-1.5509999999999999</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>903</v>
       </c>
@@ -3560,8 +3844,14 @@
         <f t="shared" si="8"/>
         <v>-1.5309999999999999</v>
       </c>
-    </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O52">
+        <v>-1.325</v>
+      </c>
+      <c r="P52">
+        <v>-1.5309999999999999</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>904</v>
       </c>
@@ -3608,8 +3898,14 @@
         <f t="shared" si="8"/>
         <v>-1.5129999999999999</v>
       </c>
-    </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O53">
+        <v>-1.331</v>
+      </c>
+      <c r="P53">
+        <v>-1.5129999999999999</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>905</v>
       </c>
@@ -3656,8 +3952,14 @@
         <f t="shared" si="8"/>
         <v>-1.474</v>
       </c>
-    </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O54">
+        <v>-1.321</v>
+      </c>
+      <c r="P54">
+        <v>-1.474</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>906</v>
       </c>
@@ -3704,8 +4006,14 @@
         <f t="shared" si="8"/>
         <v>-1.446</v>
       </c>
-    </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O55">
+        <v>-1.3140000000000001</v>
+      </c>
+      <c r="P55">
+        <v>-1.446</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>1001</v>
       </c>
@@ -3752,8 +4060,14 @@
         <f t="shared" si="8"/>
         <v>-1.6919999999999999</v>
       </c>
-    </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O56">
+        <v>-1.5640000000000001</v>
+      </c>
+      <c r="P56">
+        <v>-1.6919999999999999</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>1002</v>
       </c>
@@ -3800,8 +4114,14 @@
         <f t="shared" si="8"/>
         <v>-1.5149999999999999</v>
       </c>
-    </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O57">
+        <v>-1.3580000000000001</v>
+      </c>
+      <c r="P57">
+        <v>-1.5149999999999999</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>1003</v>
       </c>
@@ -3848,8 +4168,14 @@
         <f t="shared" si="8"/>
         <v>-1.423</v>
       </c>
-    </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O58">
+        <v>-1.1930000000000001</v>
+      </c>
+      <c r="P58">
+        <v>-1.423</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>1004</v>
       </c>
@@ -3896,8 +4222,14 @@
         <f t="shared" si="8"/>
         <v>-1.17</v>
       </c>
-    </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O59">
+        <v>-0.89500000000000002</v>
+      </c>
+      <c r="P59">
+        <v>-1.17</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>1005</v>
       </c>
@@ -3944,8 +4276,14 @@
         <f t="shared" si="8"/>
         <v>-1.3220000000000001</v>
       </c>
-    </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O60">
+        <v>-1.1759999999999999</v>
+      </c>
+      <c r="P60">
+        <v>-1.3220000000000001</v>
+      </c>
+    </row>
+    <row r="61" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>1006</v>
       </c>
@@ -3980,20 +4318,23 @@
         <f t="shared" si="3"/>
         <v>E</v>
       </c>
-      <c r="L61" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M61" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N61" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L61">
+        <v>0</v>
+      </c>
+      <c r="M61">
+        <v>0</v>
+      </c>
+      <c r="N61">
+        <v>0</v>
+      </c>
+      <c r="O61">
+        <v>0</v>
+      </c>
+      <c r="P61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>9001</v>
       </c>
@@ -4028,20 +4369,23 @@
         <f t="shared" si="3"/>
         <v>E</v>
       </c>
-      <c r="L62" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M62" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N62" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L62">
+        <v>0</v>
+      </c>
+      <c r="M62">
+        <v>0</v>
+      </c>
+      <c r="N62">
+        <v>0</v>
+      </c>
+      <c r="O62">
+        <v>0</v>
+      </c>
+      <c r="P62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>9003</v>
       </c>
@@ -4088,8 +4432,14 @@
         <f t="shared" si="8"/>
         <v>-1.86</v>
       </c>
-    </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O63">
+        <v>0</v>
+      </c>
+      <c r="P63">
+        <v>-1.86</v>
+      </c>
+    </row>
+    <row r="64" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>1101</v>
       </c>
@@ -4136,8 +4486,14 @@
         <f t="shared" si="8"/>
         <v>-1.92</v>
       </c>
-    </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O64">
+        <v>-1.911</v>
+      </c>
+      <c r="P64">
+        <v>-1.92</v>
+      </c>
+    </row>
+    <row r="65" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>1102</v>
       </c>
@@ -4184,8 +4540,14 @@
         <f t="shared" si="8"/>
         <v>-1.903</v>
       </c>
-    </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O65">
+        <v>-1.8859999999999999</v>
+      </c>
+      <c r="P65">
+        <v>-1.903</v>
+      </c>
+    </row>
+    <row r="66" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>1103</v>
       </c>
@@ -4225,15 +4587,21 @@
         <v>-1.7509999999999999</v>
       </c>
       <c r="M66">
-        <f t="shared" ref="M66:M78" si="10">VLOOKUP("Pb"&amp;$A66,yyy,6,FALSE)</f>
+        <f t="shared" ref="M66:O78" si="10">VLOOKUP("Pb"&amp;$A66,yyy,6,FALSE)</f>
         <v>-1.714</v>
       </c>
       <c r="N66">
-        <f t="shared" ref="N66:N78" si="11">VLOOKUP("Pb"&amp;$A66,yyy,7,FALSE)</f>
+        <f t="shared" ref="N66:P78" si="11">VLOOKUP("Pb"&amp;$A66,yyy,7,FALSE)</f>
         <v>-1.7649999999999999</v>
       </c>
-    </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O66">
+        <v>-1.714</v>
+      </c>
+      <c r="P66">
+        <v>-1.7649999999999999</v>
+      </c>
+    </row>
+    <row r="67" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>1104</v>
       </c>
@@ -4280,8 +4648,14 @@
         <f t="shared" si="11"/>
         <v>-1.597</v>
       </c>
-    </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O67">
+        <v>-1.47</v>
+      </c>
+      <c r="P67">
+        <v>-1.597</v>
+      </c>
+    </row>
+    <row r="68" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>1105</v>
       </c>
@@ -4328,8 +4702,14 @@
         <f t="shared" si="11"/>
         <v>-1.3460000000000001</v>
       </c>
-    </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O68">
+        <v>-1.1559999999999999</v>
+      </c>
+      <c r="P68">
+        <v>-1.3460000000000001</v>
+      </c>
+    </row>
+    <row r="69" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>1106</v>
       </c>
@@ -4376,8 +4756,14 @@
         <f t="shared" si="11"/>
         <v>-1.3680000000000001</v>
       </c>
-    </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O69">
+        <v>-1.2250000000000001</v>
+      </c>
+      <c r="P69">
+        <v>-1.3680000000000001</v>
+      </c>
+    </row>
+    <row r="70" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>1201</v>
       </c>
@@ -4424,8 +4810,14 @@
         <f t="shared" si="11"/>
         <v>-1.6140000000000001</v>
       </c>
-    </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O70">
+        <v>0</v>
+      </c>
+      <c r="P70">
+        <v>-1.6140000000000001</v>
+      </c>
+    </row>
+    <row r="71" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>1202</v>
       </c>
@@ -4472,8 +4864,14 @@
         <f t="shared" si="11"/>
         <v>-1.5640000000000001</v>
       </c>
-    </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O71">
+        <v>0</v>
+      </c>
+      <c r="P71">
+        <v>-1.5640000000000001</v>
+      </c>
+    </row>
+    <row r="72" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>1203</v>
       </c>
@@ -4520,8 +4918,14 @@
         <f t="shared" si="11"/>
         <v>-1.431</v>
       </c>
-    </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O72">
+        <v>-1.2509999999999999</v>
+      </c>
+      <c r="P72">
+        <v>-1.431</v>
+      </c>
+    </row>
+    <row r="73" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>1204</v>
       </c>
@@ -4556,20 +4960,23 @@
         <f t="shared" si="12"/>
         <v>E</v>
       </c>
-      <c r="L73" t="e">
-        <f t="shared" si="9"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M73" t="e">
-        <f t="shared" si="10"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N73" t="e">
-        <f t="shared" si="11"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L73">
+        <v>0</v>
+      </c>
+      <c r="M73">
+        <v>0</v>
+      </c>
+      <c r="N73">
+        <v>0</v>
+      </c>
+      <c r="O73">
+        <v>0</v>
+      </c>
+      <c r="P73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>1205</v>
       </c>
@@ -4604,20 +5011,23 @@
         <f t="shared" si="12"/>
         <v>E</v>
       </c>
-      <c r="L74" t="e">
-        <f t="shared" si="9"/>
-        <v>#N/A</v>
-      </c>
-      <c r="M74" t="e">
-        <f t="shared" si="10"/>
-        <v>#N/A</v>
-      </c>
-      <c r="N74" t="e">
-        <f t="shared" si="11"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L74">
+        <v>0</v>
+      </c>
+      <c r="M74">
+        <v>0</v>
+      </c>
+      <c r="N74">
+        <v>0</v>
+      </c>
+      <c r="O74">
+        <v>0</v>
+      </c>
+      <c r="P74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>1301</v>
       </c>
@@ -4664,8 +5074,14 @@
         <f t="shared" si="11"/>
         <v>-1.284</v>
       </c>
-    </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O75">
+        <v>0</v>
+      </c>
+      <c r="P75">
+        <v>-1.284</v>
+      </c>
+    </row>
+    <row r="76" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>1302</v>
       </c>
@@ -4712,8 +5128,14 @@
         <f t="shared" si="11"/>
         <v>-1.1819999999999999</v>
       </c>
-    </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O76">
+        <v>-0.88600000000000001</v>
+      </c>
+      <c r="P76">
+        <v>-1.1819999999999999</v>
+      </c>
+    </row>
+    <row r="77" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>1303</v>
       </c>
@@ -4760,8 +5182,14 @@
         <f t="shared" si="11"/>
         <v>-1.1859999999999999</v>
       </c>
-    </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O77">
+        <v>-0.93300000000000005</v>
+      </c>
+      <c r="P77">
+        <v>-1.1859999999999999</v>
+      </c>
+    </row>
+    <row r="78" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>1304</v>
       </c>
@@ -4806,6 +5234,12 @@
       </c>
       <c r="N78">
         <f t="shared" si="11"/>
+        <v>-1.3720000000000001</v>
+      </c>
+      <c r="O78">
+        <v>-1.2070000000000001</v>
+      </c>
+      <c r="P78">
         <v>-1.3720000000000001</v>
       </c>
     </row>
@@ -11062,4 +11496,3033 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7C0FFF9-DB26-954D-871D-A338BC7B0C37}">
+  <dimension ref="A1:G122"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="6" width="10.83203125" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="5">
+        <v>0</v>
+      </c>
+      <c r="B2" s="7">
+        <v>129981</v>
+      </c>
+      <c r="C2" s="7">
+        <v>475829</v>
+      </c>
+      <c r="D2" s="7">
+        <v>145.69999999999999</v>
+      </c>
+      <c r="E2" s="7">
+        <v>129837.3</v>
+      </c>
+      <c r="F2" s="7">
+        <v>475853.3</v>
+      </c>
+      <c r="G2" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="5">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7">
+        <v>129619</v>
+      </c>
+      <c r="C3" s="7">
+        <v>475921</v>
+      </c>
+      <c r="D3" s="7">
+        <v>226.6</v>
+      </c>
+      <c r="E3" s="7">
+        <v>129842.4</v>
+      </c>
+      <c r="F3" s="7">
+        <v>475883.3</v>
+      </c>
+      <c r="G3" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="5">
+        <v>2</v>
+      </c>
+      <c r="B4" s="7">
+        <v>129586</v>
+      </c>
+      <c r="C4" s="7">
+        <v>475778</v>
+      </c>
+      <c r="D4" s="7">
+        <v>235.3</v>
+      </c>
+      <c r="E4" s="7">
+        <v>129818</v>
+      </c>
+      <c r="F4" s="7">
+        <v>475738.8</v>
+      </c>
+      <c r="G4" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="5">
+        <v>3</v>
+      </c>
+      <c r="B5" s="7">
+        <v>129559</v>
+      </c>
+      <c r="C5" s="7">
+        <v>475647</v>
+      </c>
+      <c r="D5" s="7">
+        <v>240.1</v>
+      </c>
+      <c r="E5" s="7">
+        <v>129795.8</v>
+      </c>
+      <c r="F5" s="7">
+        <v>475607</v>
+      </c>
+      <c r="G5" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="5">
+        <v>4</v>
+      </c>
+      <c r="B6" s="7">
+        <v>129598</v>
+      </c>
+      <c r="C6" s="7">
+        <v>476032</v>
+      </c>
+      <c r="D6" s="7">
+        <v>265.8</v>
+      </c>
+      <c r="E6" s="7">
+        <v>129860.1</v>
+      </c>
+      <c r="F6" s="7">
+        <v>475987.7</v>
+      </c>
+      <c r="G6" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="5">
+        <v>5</v>
+      </c>
+      <c r="B7" s="7">
+        <v>129602</v>
+      </c>
+      <c r="C7" s="7">
+        <v>476057</v>
+      </c>
+      <c r="D7" s="7">
+        <v>266</v>
+      </c>
+      <c r="E7" s="7">
+        <v>129864.3</v>
+      </c>
+      <c r="F7" s="7">
+        <v>476012.7</v>
+      </c>
+      <c r="G7" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="5">
+        <v>6</v>
+      </c>
+      <c r="B8" s="7">
+        <v>129570</v>
+      </c>
+      <c r="C8" s="7">
+        <v>475998</v>
+      </c>
+      <c r="D8" s="7">
+        <v>287.7</v>
+      </c>
+      <c r="E8" s="7">
+        <v>129853.7</v>
+      </c>
+      <c r="F8" s="7">
+        <v>475950.1</v>
+      </c>
+      <c r="G8" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="5">
+        <v>7</v>
+      </c>
+      <c r="B9" s="7">
+        <v>129551</v>
+      </c>
+      <c r="C9" s="7">
+        <v>475915</v>
+      </c>
+      <c r="D9" s="7">
+        <v>292.60000000000002</v>
+      </c>
+      <c r="E9" s="7">
+        <v>129839.5</v>
+      </c>
+      <c r="F9" s="7">
+        <v>475866.3</v>
+      </c>
+      <c r="G9" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="5">
+        <v>8</v>
+      </c>
+      <c r="B10" s="7">
+        <v>129503</v>
+      </c>
+      <c r="C10" s="7">
+        <v>475910</v>
+      </c>
+      <c r="D10" s="7">
+        <v>339.1</v>
+      </c>
+      <c r="E10" s="7">
+        <v>129837.4</v>
+      </c>
+      <c r="F10" s="7">
+        <v>475853.5</v>
+      </c>
+      <c r="G10" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="5">
+        <v>9</v>
+      </c>
+      <c r="B11" s="7">
+        <v>129464</v>
+      </c>
+      <c r="C11" s="7">
+        <v>475696</v>
+      </c>
+      <c r="D11" s="7">
+        <v>341.9</v>
+      </c>
+      <c r="E11" s="7">
+        <v>129801.2</v>
+      </c>
+      <c r="F11" s="7">
+        <v>475639.1</v>
+      </c>
+      <c r="G11" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="5">
+        <v>10</v>
+      </c>
+      <c r="B12" s="7">
+        <v>129469</v>
+      </c>
+      <c r="C12" s="7">
+        <v>475748</v>
+      </c>
+      <c r="D12" s="7">
+        <v>345.7</v>
+      </c>
+      <c r="E12" s="7">
+        <v>129809.8</v>
+      </c>
+      <c r="F12" s="7">
+        <v>475690.4</v>
+      </c>
+      <c r="G12" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="5">
+        <v>11</v>
+      </c>
+      <c r="B13" s="7">
+        <v>129462</v>
+      </c>
+      <c r="C13" s="7">
+        <v>475907</v>
+      </c>
+      <c r="D13" s="7">
+        <v>379.1</v>
+      </c>
+      <c r="E13" s="7">
+        <v>129835.8</v>
+      </c>
+      <c r="F13" s="7">
+        <v>475843.9</v>
+      </c>
+      <c r="G13" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="5">
+        <v>12</v>
+      </c>
+      <c r="B14" s="7">
+        <v>129450</v>
+      </c>
+      <c r="C14" s="7">
+        <v>475856</v>
+      </c>
+      <c r="D14" s="7">
+        <v>382.4</v>
+      </c>
+      <c r="E14" s="7">
+        <v>129827.1</v>
+      </c>
+      <c r="F14" s="7">
+        <v>475792.3</v>
+      </c>
+      <c r="G14" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" s="5">
+        <v>13</v>
+      </c>
+      <c r="B15" s="7">
+        <v>129404</v>
+      </c>
+      <c r="C15" s="7">
+        <v>475743</v>
+      </c>
+      <c r="D15" s="7">
+        <v>408.9</v>
+      </c>
+      <c r="E15" s="7">
+        <v>129807.2</v>
+      </c>
+      <c r="F15" s="7">
+        <v>475674.9</v>
+      </c>
+      <c r="G15" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="5">
+        <v>14</v>
+      </c>
+      <c r="B16" s="7">
+        <v>129427</v>
+      </c>
+      <c r="C16" s="7">
+        <v>475929</v>
+      </c>
+      <c r="D16" s="7">
+        <v>417.2</v>
+      </c>
+      <c r="E16" s="7">
+        <v>129838.39999999999</v>
+      </c>
+      <c r="F16" s="7">
+        <v>475859.5</v>
+      </c>
+      <c r="G16" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" s="5">
+        <v>15</v>
+      </c>
+      <c r="B17" s="7">
+        <v>129366</v>
+      </c>
+      <c r="C17" s="7">
+        <v>475739</v>
+      </c>
+      <c r="D17" s="7">
+        <v>445.7</v>
+      </c>
+      <c r="E17" s="7">
+        <v>129805.5</v>
+      </c>
+      <c r="F17" s="7">
+        <v>475664.8</v>
+      </c>
+      <c r="G17" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="5">
+        <v>16</v>
+      </c>
+      <c r="B18" s="7">
+        <v>129408</v>
+      </c>
+      <c r="C18" s="7">
+        <v>476034</v>
+      </c>
+      <c r="D18" s="7">
+        <v>453.4</v>
+      </c>
+      <c r="E18" s="7">
+        <v>129855.1</v>
+      </c>
+      <c r="F18" s="7">
+        <v>475958.5</v>
+      </c>
+      <c r="G18" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" s="5">
+        <v>17</v>
+      </c>
+      <c r="B19" s="7">
+        <v>129405</v>
+      </c>
+      <c r="C19" s="7">
+        <v>476105</v>
+      </c>
+      <c r="D19" s="7">
+        <v>468.2</v>
+      </c>
+      <c r="E19" s="7">
+        <v>129866.7</v>
+      </c>
+      <c r="F19" s="7">
+        <v>476027</v>
+      </c>
+      <c r="G19" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" s="5">
+        <v>18</v>
+      </c>
+      <c r="B20" s="7">
+        <v>129332</v>
+      </c>
+      <c r="C20" s="7">
+        <v>475738</v>
+      </c>
+      <c r="D20" s="7">
+        <v>479.1</v>
+      </c>
+      <c r="E20" s="7">
+        <v>129804.4</v>
+      </c>
+      <c r="F20" s="7">
+        <v>475658.2</v>
+      </c>
+      <c r="G20" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" s="5">
+        <v>19</v>
+      </c>
+      <c r="B21" s="7">
+        <v>129398</v>
+      </c>
+      <c r="C21" s="7">
+        <v>476168</v>
+      </c>
+      <c r="D21" s="7">
+        <v>485.6</v>
+      </c>
+      <c r="E21" s="7">
+        <v>129876.8</v>
+      </c>
+      <c r="F21" s="7">
+        <v>476087.1</v>
+      </c>
+      <c r="G21" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" s="5">
+        <v>20</v>
+      </c>
+      <c r="B22" s="7">
+        <v>129359</v>
+      </c>
+      <c r="C22" s="7">
+        <v>476031</v>
+      </c>
+      <c r="D22" s="7">
+        <v>501.3</v>
+      </c>
+      <c r="E22" s="7">
+        <v>129853.3</v>
+      </c>
+      <c r="F22" s="7">
+        <v>475947.5</v>
+      </c>
+      <c r="G22" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" s="5">
+        <v>21</v>
+      </c>
+      <c r="B23" s="7">
+        <v>129301</v>
+      </c>
+      <c r="C23" s="7">
+        <v>475730</v>
+      </c>
+      <c r="D23" s="7">
+        <v>508.3</v>
+      </c>
+      <c r="E23" s="7">
+        <v>129802.2</v>
+      </c>
+      <c r="F23" s="7">
+        <v>475645.3</v>
+      </c>
+      <c r="G23" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" s="5">
+        <v>22</v>
+      </c>
+      <c r="B24" s="7">
+        <v>129304</v>
+      </c>
+      <c r="C24" s="7">
+        <v>475876</v>
+      </c>
+      <c r="D24" s="7">
+        <v>529.70000000000005</v>
+      </c>
+      <c r="E24" s="7">
+        <v>129826.3</v>
+      </c>
+      <c r="F24" s="7">
+        <v>475787.8</v>
+      </c>
+      <c r="G24" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" s="5">
+        <v>23</v>
+      </c>
+      <c r="B25" s="7">
+        <v>129304</v>
+      </c>
+      <c r="C25" s="7">
+        <v>475932</v>
+      </c>
+      <c r="D25" s="7">
+        <v>539</v>
+      </c>
+      <c r="E25" s="7">
+        <v>129835.5</v>
+      </c>
+      <c r="F25" s="7">
+        <v>475842.2</v>
+      </c>
+      <c r="G25" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" s="5">
+        <v>24</v>
+      </c>
+      <c r="B26" s="7">
+        <v>129310</v>
+      </c>
+      <c r="C26" s="7">
+        <v>476030</v>
+      </c>
+      <c r="D26" s="7">
+        <v>549.4</v>
+      </c>
+      <c r="E26" s="7">
+        <v>129851.7</v>
+      </c>
+      <c r="F26" s="7">
+        <v>475938.5</v>
+      </c>
+      <c r="G26" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A27" s="5">
+        <v>25</v>
+      </c>
+      <c r="B27" s="7">
+        <v>129232</v>
+      </c>
+      <c r="C27" s="7">
+        <v>475746</v>
+      </c>
+      <c r="D27" s="7">
+        <v>579</v>
+      </c>
+      <c r="E27" s="7">
+        <v>129802.9</v>
+      </c>
+      <c r="F27" s="7">
+        <v>475649.6</v>
+      </c>
+      <c r="G27" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A28" s="5">
+        <v>26</v>
+      </c>
+      <c r="B28" s="7">
+        <v>129209</v>
+      </c>
+      <c r="C28" s="7">
+        <v>476045</v>
+      </c>
+      <c r="D28" s="7">
+        <v>651.5</v>
+      </c>
+      <c r="E28" s="7">
+        <v>129851.4</v>
+      </c>
+      <c r="F28" s="7">
+        <v>475936.5</v>
+      </c>
+      <c r="G28" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A29" s="5">
+        <v>27</v>
+      </c>
+      <c r="B29" s="7">
+        <v>129158</v>
+      </c>
+      <c r="C29" s="7">
+        <v>475768</v>
+      </c>
+      <c r="D29" s="7">
+        <v>655.7</v>
+      </c>
+      <c r="E29" s="7">
+        <v>129804.5</v>
+      </c>
+      <c r="F29" s="7">
+        <v>475658.8</v>
+      </c>
+      <c r="G29" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A30" s="5">
+        <v>28</v>
+      </c>
+      <c r="B30" s="7">
+        <v>129186</v>
+      </c>
+      <c r="C30" s="7">
+        <v>475942</v>
+      </c>
+      <c r="D30" s="7">
+        <v>657</v>
+      </c>
+      <c r="E30" s="7">
+        <v>129833.9</v>
+      </c>
+      <c r="F30" s="7">
+        <v>475832.6</v>
+      </c>
+      <c r="G30" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A31" s="5">
+        <v>29</v>
+      </c>
+      <c r="B31" s="7">
+        <v>129186</v>
+      </c>
+      <c r="C31" s="7">
+        <v>475995</v>
+      </c>
+      <c r="D31" s="7">
+        <v>665.9</v>
+      </c>
+      <c r="E31" s="7">
+        <v>129842.6</v>
+      </c>
+      <c r="F31" s="7">
+        <v>475884.1</v>
+      </c>
+      <c r="G31" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A32" s="5">
+        <v>30</v>
+      </c>
+      <c r="B32" s="7">
+        <v>129161</v>
+      </c>
+      <c r="C32" s="7">
+        <v>475905</v>
+      </c>
+      <c r="D32" s="7">
+        <v>675.5</v>
+      </c>
+      <c r="E32" s="7">
+        <v>129827.1</v>
+      </c>
+      <c r="F32" s="7">
+        <v>475792.5</v>
+      </c>
+      <c r="G32" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A33" s="5">
+        <v>31</v>
+      </c>
+      <c r="B33" s="7">
+        <v>129714</v>
+      </c>
+      <c r="C33" s="7">
+        <v>475490</v>
+      </c>
+      <c r="D33" s="7">
+        <v>61.1</v>
+      </c>
+      <c r="E33" s="7">
+        <v>129774.3</v>
+      </c>
+      <c r="F33" s="7">
+        <v>475479.8</v>
+      </c>
+      <c r="G33" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A34" s="5">
+        <v>32</v>
+      </c>
+      <c r="B34" s="7">
+        <v>129683</v>
+      </c>
+      <c r="C34" s="7">
+        <v>475385</v>
+      </c>
+      <c r="D34" s="7">
+        <v>74.2</v>
+      </c>
+      <c r="E34" s="7">
+        <v>129756.2</v>
+      </c>
+      <c r="F34" s="7">
+        <v>475372.6</v>
+      </c>
+      <c r="G34" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A35" s="5">
+        <v>33</v>
+      </c>
+      <c r="B35" s="7">
+        <v>129668</v>
+      </c>
+      <c r="C35" s="7">
+        <v>475328</v>
+      </c>
+      <c r="D35" s="7">
+        <v>79.5</v>
+      </c>
+      <c r="E35" s="7">
+        <v>129746.4</v>
+      </c>
+      <c r="F35" s="7">
+        <v>475314.8</v>
+      </c>
+      <c r="G35" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A36" s="5">
+        <v>34</v>
+      </c>
+      <c r="B36" s="7">
+        <v>129718</v>
+      </c>
+      <c r="C36" s="7">
+        <v>475636</v>
+      </c>
+      <c r="D36" s="7">
+        <v>81.5</v>
+      </c>
+      <c r="E36" s="7">
+        <v>129798.39999999999</v>
+      </c>
+      <c r="F36" s="7">
+        <v>475622.40000000002</v>
+      </c>
+      <c r="G36" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A37" s="5">
+        <v>35</v>
+      </c>
+      <c r="B37" s="7">
+        <v>129714</v>
+      </c>
+      <c r="C37" s="7">
+        <v>475616</v>
+      </c>
+      <c r="D37" s="7">
+        <v>82.1</v>
+      </c>
+      <c r="E37" s="7">
+        <v>129795</v>
+      </c>
+      <c r="F37" s="7">
+        <v>475602.3</v>
+      </c>
+      <c r="G37" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A38" s="5">
+        <v>36</v>
+      </c>
+      <c r="B38" s="7">
+        <v>129873</v>
+      </c>
+      <c r="C38" s="7">
+        <v>475466</v>
+      </c>
+      <c r="D38" s="7">
+        <v>99.6</v>
+      </c>
+      <c r="E38" s="7">
+        <v>129774.7</v>
+      </c>
+      <c r="F38" s="7">
+        <v>475482.6</v>
+      </c>
+      <c r="G38" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A39" s="5">
+        <v>37</v>
+      </c>
+      <c r="B39" s="7">
+        <v>129643</v>
+      </c>
+      <c r="C39" s="7">
+        <v>475311</v>
+      </c>
+      <c r="D39" s="7">
+        <v>101.3</v>
+      </c>
+      <c r="E39" s="7">
+        <v>129742.9</v>
+      </c>
+      <c r="F39" s="7">
+        <v>475294.1</v>
+      </c>
+      <c r="G39" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A40" s="5">
+        <v>38</v>
+      </c>
+      <c r="B40" s="7">
+        <v>129842</v>
+      </c>
+      <c r="C40" s="7">
+        <v>475269</v>
+      </c>
+      <c r="D40" s="7">
+        <v>101.9</v>
+      </c>
+      <c r="E40" s="7">
+        <v>129741.5</v>
+      </c>
+      <c r="F40" s="7">
+        <v>475286</v>
+      </c>
+      <c r="G40" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A41" s="5">
+        <v>39</v>
+      </c>
+      <c r="B41" s="7">
+        <v>129862</v>
+      </c>
+      <c r="C41" s="7">
+        <v>475337</v>
+      </c>
+      <c r="D41" s="7">
+        <v>110.3</v>
+      </c>
+      <c r="E41" s="7">
+        <v>129753.3</v>
+      </c>
+      <c r="F41" s="7">
+        <v>475355.4</v>
+      </c>
+      <c r="G41" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A42" s="5">
+        <v>40</v>
+      </c>
+      <c r="B42" s="7">
+        <v>129882</v>
+      </c>
+      <c r="C42" s="7">
+        <v>475422</v>
+      </c>
+      <c r="D42" s="7">
+        <v>115.9</v>
+      </c>
+      <c r="E42" s="7">
+        <v>129767.8</v>
+      </c>
+      <c r="F42" s="7">
+        <v>475441.3</v>
+      </c>
+      <c r="G42" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A43" s="5">
+        <v>41</v>
+      </c>
+      <c r="B43" s="7">
+        <v>129900</v>
+      </c>
+      <c r="C43" s="7">
+        <v>475479</v>
+      </c>
+      <c r="D43" s="7">
+        <v>124.1</v>
+      </c>
+      <c r="E43" s="7">
+        <v>129777.60000000001</v>
+      </c>
+      <c r="F43" s="7">
+        <v>475499.7</v>
+      </c>
+      <c r="G43" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A44" s="5">
+        <v>42</v>
+      </c>
+      <c r="B44" s="7">
+        <v>129855</v>
+      </c>
+      <c r="C44" s="7">
+        <v>475210</v>
+      </c>
+      <c r="D44" s="7">
+        <v>124.5</v>
+      </c>
+      <c r="E44" s="7">
+        <v>129732.2</v>
+      </c>
+      <c r="F44" s="7">
+        <v>475230.7</v>
+      </c>
+      <c r="G44" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A45" s="5">
+        <v>43</v>
+      </c>
+      <c r="B45" s="7">
+        <v>129923</v>
+      </c>
+      <c r="C45" s="7">
+        <v>475596</v>
+      </c>
+      <c r="D45" s="7">
+        <v>127.3</v>
+      </c>
+      <c r="E45" s="7">
+        <v>129797.5</v>
+      </c>
+      <c r="F45" s="7">
+        <v>475617.2</v>
+      </c>
+      <c r="G45" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A46" s="5">
+        <v>44</v>
+      </c>
+      <c r="B46" s="7">
+        <v>129644</v>
+      </c>
+      <c r="C46" s="7">
+        <v>475500</v>
+      </c>
+      <c r="D46" s="7">
+        <v>131.80000000000001</v>
+      </c>
+      <c r="E46" s="7">
+        <v>129774</v>
+      </c>
+      <c r="F46" s="7">
+        <v>475478</v>
+      </c>
+      <c r="G46" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A47" s="5">
+        <v>45</v>
+      </c>
+      <c r="B47" s="7">
+        <v>129607</v>
+      </c>
+      <c r="C47" s="7">
+        <v>475330</v>
+      </c>
+      <c r="D47" s="7">
+        <v>140</v>
+      </c>
+      <c r="E47" s="7">
+        <v>129745</v>
+      </c>
+      <c r="F47" s="7">
+        <v>475306.7</v>
+      </c>
+      <c r="G47" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A48" s="5">
+        <v>46</v>
+      </c>
+      <c r="B48" s="7">
+        <v>129887</v>
+      </c>
+      <c r="C48" s="7">
+        <v>475277</v>
+      </c>
+      <c r="D48" s="7">
+        <v>144.9</v>
+      </c>
+      <c r="E48" s="7">
+        <v>129744.1</v>
+      </c>
+      <c r="F48" s="7">
+        <v>475301.1</v>
+      </c>
+      <c r="G48" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A49" s="5">
+        <v>47</v>
+      </c>
+      <c r="B49" s="7">
+        <v>129607</v>
+      </c>
+      <c r="C49" s="7">
+        <v>475378</v>
+      </c>
+      <c r="D49" s="7">
+        <v>148</v>
+      </c>
+      <c r="E49" s="7">
+        <v>129752.9</v>
+      </c>
+      <c r="F49" s="7">
+        <v>475353.4</v>
+      </c>
+      <c r="G49" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A50" s="5">
+        <v>48</v>
+      </c>
+      <c r="B50" s="7">
+        <v>129626</v>
+      </c>
+      <c r="C50" s="7">
+        <v>475538</v>
+      </c>
+      <c r="D50" s="7">
+        <v>155.9</v>
+      </c>
+      <c r="E50" s="7">
+        <v>129779.7</v>
+      </c>
+      <c r="F50" s="7">
+        <v>475512</v>
+      </c>
+      <c r="G50" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A51" s="5">
+        <v>49</v>
+      </c>
+      <c r="B51" s="7">
+        <v>129935</v>
+      </c>
+      <c r="C51" s="7">
+        <v>475489</v>
+      </c>
+      <c r="D51" s="7">
+        <v>157</v>
+      </c>
+      <c r="E51" s="7">
+        <v>129780.2</v>
+      </c>
+      <c r="F51" s="7">
+        <v>475515.1</v>
+      </c>
+      <c r="G51" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A52" s="5">
+        <v>50</v>
+      </c>
+      <c r="B52" s="7">
+        <v>129575</v>
+      </c>
+      <c r="C52" s="7">
+        <v>475303</v>
+      </c>
+      <c r="D52" s="7">
+        <v>167</v>
+      </c>
+      <c r="E52" s="7">
+        <v>129739.7</v>
+      </c>
+      <c r="F52" s="7">
+        <v>475275.2</v>
+      </c>
+      <c r="G52" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A53" s="5">
+        <v>51</v>
+      </c>
+      <c r="B53" s="7">
+        <v>129971</v>
+      </c>
+      <c r="C53" s="7">
+        <v>475634</v>
+      </c>
+      <c r="D53" s="7">
+        <v>168.3</v>
+      </c>
+      <c r="E53" s="7">
+        <v>129805</v>
+      </c>
+      <c r="F53" s="7">
+        <v>475662</v>
+      </c>
+      <c r="G53" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A54" s="5">
+        <v>52</v>
+      </c>
+      <c r="B54" s="7">
+        <v>129544</v>
+      </c>
+      <c r="C54" s="7">
+        <v>475257</v>
+      </c>
+      <c r="D54" s="7">
+        <v>190</v>
+      </c>
+      <c r="E54" s="7">
+        <v>129731.3</v>
+      </c>
+      <c r="F54" s="7">
+        <v>475225.4</v>
+      </c>
+      <c r="G54" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A55" s="5">
+        <v>53</v>
+      </c>
+      <c r="B55" s="7">
+        <v>129956</v>
+      </c>
+      <c r="C55" s="7">
+        <v>475354</v>
+      </c>
+      <c r="D55" s="7">
+        <v>200.1</v>
+      </c>
+      <c r="E55" s="7">
+        <v>129758.7</v>
+      </c>
+      <c r="F55" s="7">
+        <v>475387.3</v>
+      </c>
+      <c r="G55" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A56" s="5">
+        <v>54</v>
+      </c>
+      <c r="B56" s="7">
+        <v>129569</v>
+      </c>
+      <c r="C56" s="7">
+        <v>475520</v>
+      </c>
+      <c r="D56" s="7">
+        <v>209.1</v>
+      </c>
+      <c r="E56" s="7">
+        <v>129775.2</v>
+      </c>
+      <c r="F56" s="7">
+        <v>475485.2</v>
+      </c>
+      <c r="G56" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A57" s="5">
+        <v>55</v>
+      </c>
+      <c r="B57" s="7">
+        <v>129526</v>
+      </c>
+      <c r="C57" s="7">
+        <v>475341</v>
+      </c>
+      <c r="D57" s="7">
+        <v>221.7</v>
+      </c>
+      <c r="E57" s="7">
+        <v>129744.6</v>
+      </c>
+      <c r="F57" s="7">
+        <v>475304.1</v>
+      </c>
+      <c r="G57" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A58" s="5">
+        <v>56</v>
+      </c>
+      <c r="B58" s="7">
+        <v>129488</v>
+      </c>
+      <c r="C58" s="7">
+        <v>475256</v>
+      </c>
+      <c r="D58" s="7">
+        <v>245</v>
+      </c>
+      <c r="E58" s="7">
+        <v>129729.60000000001</v>
+      </c>
+      <c r="F58" s="7">
+        <v>475215.2</v>
+      </c>
+      <c r="G58" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A59" s="5">
+        <v>57</v>
+      </c>
+      <c r="B59" s="7">
+        <v>129473</v>
+      </c>
+      <c r="C59" s="7">
+        <v>475222</v>
+      </c>
+      <c r="D59" s="7">
+        <v>254.1</v>
+      </c>
+      <c r="E59" s="7">
+        <v>129723.6</v>
+      </c>
+      <c r="F59" s="7">
+        <v>475179.7</v>
+      </c>
+      <c r="G59" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A60" s="5">
+        <v>58</v>
+      </c>
+      <c r="B60" s="7">
+        <v>129993</v>
+      </c>
+      <c r="C60" s="7">
+        <v>475245</v>
+      </c>
+      <c r="D60" s="7">
+        <v>254.8</v>
+      </c>
+      <c r="E60" s="7">
+        <v>129741.8</v>
+      </c>
+      <c r="F60" s="7">
+        <v>475287.4</v>
+      </c>
+      <c r="G60" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A61" s="5">
+        <v>59</v>
+      </c>
+      <c r="B61" s="7">
+        <v>129481</v>
+      </c>
+      <c r="C61" s="7">
+        <v>475320</v>
+      </c>
+      <c r="D61" s="7">
+        <v>262.60000000000002</v>
+      </c>
+      <c r="E61" s="7">
+        <v>129739.9</v>
+      </c>
+      <c r="F61" s="7">
+        <v>475276.3</v>
+      </c>
+      <c r="G61" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A62" s="5">
+        <v>60</v>
+      </c>
+      <c r="B62" s="7">
+        <v>129490</v>
+      </c>
+      <c r="C62" s="7">
+        <v>475387</v>
+      </c>
+      <c r="D62" s="7">
+        <v>264.8</v>
+      </c>
+      <c r="E62" s="7">
+        <v>129751.1</v>
+      </c>
+      <c r="F62" s="7">
+        <v>475342.9</v>
+      </c>
+      <c r="G62" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A63" s="5">
+        <v>61</v>
+      </c>
+      <c r="B63" s="7">
+        <v>130067</v>
+      </c>
+      <c r="C63" s="7">
+        <v>475607</v>
+      </c>
+      <c r="D63" s="7">
+        <v>267.5</v>
+      </c>
+      <c r="E63" s="7">
+        <v>129803.3</v>
+      </c>
+      <c r="F63" s="7">
+        <v>475651.5</v>
+      </c>
+      <c r="G63" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A64" s="5">
+        <v>62</v>
+      </c>
+      <c r="B64" s="7">
+        <v>129494</v>
+      </c>
+      <c r="C64" s="7">
+        <v>475443</v>
+      </c>
+      <c r="D64" s="7">
+        <v>270.2</v>
+      </c>
+      <c r="E64" s="7">
+        <v>129760.5</v>
+      </c>
+      <c r="F64" s="7">
+        <v>475398</v>
+      </c>
+      <c r="G64" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A65" s="5">
+        <v>63</v>
+      </c>
+      <c r="B65" s="7">
+        <v>130006</v>
+      </c>
+      <c r="C65" s="7">
+        <v>475226</v>
+      </c>
+      <c r="D65" s="7">
+        <v>270.8</v>
+      </c>
+      <c r="E65" s="7">
+        <v>129739</v>
+      </c>
+      <c r="F65" s="7">
+        <v>475271.1</v>
+      </c>
+      <c r="G65" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A66" s="5">
+        <v>64</v>
+      </c>
+      <c r="B66" s="7">
+        <v>129501</v>
+      </c>
+      <c r="C66" s="7">
+        <v>475495</v>
+      </c>
+      <c r="D66" s="7">
+        <v>272</v>
+      </c>
+      <c r="E66" s="7">
+        <v>129769.2</v>
+      </c>
+      <c r="F66" s="7">
+        <v>475449.7</v>
+      </c>
+      <c r="G66" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A67" s="5">
+        <v>65</v>
+      </c>
+      <c r="B67" s="7">
+        <v>130084</v>
+      </c>
+      <c r="C67" s="7">
+        <v>475532</v>
+      </c>
+      <c r="D67" s="7">
+        <v>296.7</v>
+      </c>
+      <c r="E67" s="7">
+        <v>129791.4</v>
+      </c>
+      <c r="F67" s="7">
+        <v>475581.4</v>
+      </c>
+      <c r="G67" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A68" s="5">
+        <v>66</v>
+      </c>
+      <c r="B68" s="7">
+        <v>130109</v>
+      </c>
+      <c r="C68" s="7">
+        <v>475599</v>
+      </c>
+      <c r="D68" s="7">
+        <v>310.2</v>
+      </c>
+      <c r="E68" s="7">
+        <v>129803.1</v>
+      </c>
+      <c r="F68" s="7">
+        <v>475650.7</v>
+      </c>
+      <c r="G68" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A69" s="5">
+        <v>67</v>
+      </c>
+      <c r="B69" s="7">
+        <v>130070</v>
+      </c>
+      <c r="C69" s="7">
+        <v>475241</v>
+      </c>
+      <c r="D69" s="7">
+        <v>331.4</v>
+      </c>
+      <c r="E69" s="7">
+        <v>129743.3</v>
+      </c>
+      <c r="F69" s="7">
+        <v>475296.2</v>
+      </c>
+      <c r="G69" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A70" s="5">
+        <v>68</v>
+      </c>
+      <c r="B70" s="7">
+        <v>129440</v>
+      </c>
+      <c r="C70" s="7">
+        <v>475492</v>
+      </c>
+      <c r="D70" s="7">
+        <v>331.6</v>
+      </c>
+      <c r="E70" s="7">
+        <v>129767</v>
+      </c>
+      <c r="F70" s="7">
+        <v>475436.79999999999</v>
+      </c>
+      <c r="G70" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A71" s="5">
+        <v>69</v>
+      </c>
+      <c r="B71" s="7">
+        <v>129362</v>
+      </c>
+      <c r="C71" s="7">
+        <v>475439</v>
+      </c>
+      <c r="D71" s="7">
+        <v>399.7</v>
+      </c>
+      <c r="E71" s="7">
+        <v>129756.1</v>
+      </c>
+      <c r="F71" s="7">
+        <v>475372.4</v>
+      </c>
+      <c r="G71" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A72" s="5">
+        <v>70</v>
+      </c>
+      <c r="B72" s="7">
+        <v>129293</v>
+      </c>
+      <c r="C72" s="7">
+        <v>475285</v>
+      </c>
+      <c r="D72" s="7">
+        <v>442.1</v>
+      </c>
+      <c r="E72" s="7">
+        <v>129728.9</v>
+      </c>
+      <c r="F72" s="7">
+        <v>475211.4</v>
+      </c>
+      <c r="G72" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A73" s="5">
+        <v>71</v>
+      </c>
+      <c r="B73" s="7">
+        <v>129257</v>
+      </c>
+      <c r="C73" s="7">
+        <v>475265</v>
+      </c>
+      <c r="D73" s="7">
+        <v>474.3</v>
+      </c>
+      <c r="E73" s="7">
+        <v>129724.7</v>
+      </c>
+      <c r="F73" s="7">
+        <v>475186</v>
+      </c>
+      <c r="G73" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A74" s="5">
+        <v>72</v>
+      </c>
+      <c r="B74" s="7">
+        <v>129811</v>
+      </c>
+      <c r="C74" s="7">
+        <v>475136</v>
+      </c>
+      <c r="D74" s="7">
+        <v>93.5</v>
+      </c>
+      <c r="E74" s="7">
+        <v>129718.8</v>
+      </c>
+      <c r="F74" s="7">
+        <v>475151.6</v>
+      </c>
+      <c r="G74" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A75" s="5">
+        <v>73</v>
+      </c>
+      <c r="B75" s="7">
+        <v>129778</v>
+      </c>
+      <c r="C75" s="7">
+        <v>474923</v>
+      </c>
+      <c r="D75" s="7">
+        <v>96.4</v>
+      </c>
+      <c r="E75" s="7">
+        <v>129682.9</v>
+      </c>
+      <c r="F75" s="7">
+        <v>474939.1</v>
+      </c>
+      <c r="G75" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A76" s="5">
+        <v>74</v>
+      </c>
+      <c r="B76" s="7">
+        <v>129812</v>
+      </c>
+      <c r="C76" s="7">
+        <v>474987</v>
+      </c>
+      <c r="D76" s="7">
+        <v>119.3</v>
+      </c>
+      <c r="E76" s="7">
+        <v>129694.39999999999</v>
+      </c>
+      <c r="F76" s="7">
+        <v>475006.9</v>
+      </c>
+      <c r="G76" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A77" s="5">
+        <v>75</v>
+      </c>
+      <c r="B77" s="7">
+        <v>129760</v>
+      </c>
+      <c r="C77" s="7">
+        <v>474653</v>
+      </c>
+      <c r="D77" s="7">
+        <v>123.9</v>
+      </c>
+      <c r="E77" s="7">
+        <v>129637.9</v>
+      </c>
+      <c r="F77" s="7">
+        <v>474674.1</v>
+      </c>
+      <c r="G77" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A78" s="5">
+        <v>76</v>
+      </c>
+      <c r="B78" s="7">
+        <v>129833</v>
+      </c>
+      <c r="C78" s="7">
+        <v>475080</v>
+      </c>
+      <c r="D78" s="7">
+        <v>124.5</v>
+      </c>
+      <c r="E78" s="7">
+        <v>129710.2</v>
+      </c>
+      <c r="F78" s="7">
+        <v>475100.7</v>
+      </c>
+      <c r="G78" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A79" s="5">
+        <v>77</v>
+      </c>
+      <c r="B79" s="7">
+        <v>129856</v>
+      </c>
+      <c r="C79" s="7">
+        <v>475117</v>
+      </c>
+      <c r="D79" s="7">
+        <v>141</v>
+      </c>
+      <c r="E79" s="7">
+        <v>129717</v>
+      </c>
+      <c r="F79" s="7">
+        <v>475140.5</v>
+      </c>
+      <c r="G79" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A80" s="5">
+        <v>78</v>
+      </c>
+      <c r="B80" s="7">
+        <v>129541</v>
+      </c>
+      <c r="C80" s="7">
+        <v>475052</v>
+      </c>
+      <c r="D80" s="7">
+        <v>158.80000000000001</v>
+      </c>
+      <c r="E80" s="7">
+        <v>129697.60000000001</v>
+      </c>
+      <c r="F80" s="7">
+        <v>475025.6</v>
+      </c>
+      <c r="G80" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A81" s="5">
+        <v>79</v>
+      </c>
+      <c r="B81" s="7">
+        <v>129862</v>
+      </c>
+      <c r="C81" s="7">
+        <v>475037</v>
+      </c>
+      <c r="D81" s="7">
+        <v>160.19999999999999</v>
+      </c>
+      <c r="E81" s="7">
+        <v>129704</v>
+      </c>
+      <c r="F81" s="7">
+        <v>475063.7</v>
+      </c>
+      <c r="G81" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A82" s="5">
+        <v>80</v>
+      </c>
+      <c r="B82" s="7">
+        <v>129866</v>
+      </c>
+      <c r="C82" s="7">
+        <v>474988</v>
+      </c>
+      <c r="D82" s="7">
+        <v>172.3</v>
+      </c>
+      <c r="E82" s="7">
+        <v>129696.1</v>
+      </c>
+      <c r="F82" s="7">
+        <v>475016.7</v>
+      </c>
+      <c r="G82" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A83" s="5">
+        <v>81</v>
+      </c>
+      <c r="B83" s="7">
+        <v>129541</v>
+      </c>
+      <c r="C83" s="7">
+        <v>475142</v>
+      </c>
+      <c r="D83" s="7">
+        <v>173.8</v>
+      </c>
+      <c r="E83" s="7">
+        <v>129712.3</v>
+      </c>
+      <c r="F83" s="7">
+        <v>475113.1</v>
+      </c>
+      <c r="G83" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A84" s="5">
+        <v>82</v>
+      </c>
+      <c r="B84" s="7">
+        <v>129502</v>
+      </c>
+      <c r="C84" s="7">
+        <v>475116</v>
+      </c>
+      <c r="D84" s="7">
+        <v>207.9</v>
+      </c>
+      <c r="E84" s="7">
+        <v>129707</v>
+      </c>
+      <c r="F84" s="7">
+        <v>475081.4</v>
+      </c>
+      <c r="G84" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A85" s="5">
+        <v>83</v>
+      </c>
+      <c r="B85" s="7">
+        <v>129493</v>
+      </c>
+      <c r="C85" s="7">
+        <v>475075</v>
+      </c>
+      <c r="D85" s="7">
+        <v>209.9</v>
+      </c>
+      <c r="E85" s="7">
+        <v>129700</v>
+      </c>
+      <c r="F85" s="7">
+        <v>475040</v>
+      </c>
+      <c r="G85" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A86" s="5">
+        <v>84</v>
+      </c>
+      <c r="B86" s="7">
+        <v>129503</v>
+      </c>
+      <c r="C86" s="7">
+        <v>475170</v>
+      </c>
+      <c r="D86" s="7">
+        <v>215.9</v>
+      </c>
+      <c r="E86" s="7">
+        <v>129715.9</v>
+      </c>
+      <c r="F86" s="7">
+        <v>475134</v>
+      </c>
+      <c r="G86" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A87" s="5">
+        <v>85</v>
+      </c>
+      <c r="B87" s="7">
+        <v>129857</v>
+      </c>
+      <c r="C87" s="7">
+        <v>474650</v>
+      </c>
+      <c r="D87" s="7">
+        <v>220</v>
+      </c>
+      <c r="E87" s="7">
+        <v>129640.2</v>
+      </c>
+      <c r="F87" s="7">
+        <v>474687.5</v>
+      </c>
+      <c r="G87" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A88" s="5">
+        <v>86</v>
+      </c>
+      <c r="B88" s="7">
+        <v>129448</v>
+      </c>
+      <c r="C88" s="7">
+        <v>474892</v>
+      </c>
+      <c r="D88" s="7">
+        <v>223.8</v>
+      </c>
+      <c r="E88" s="7">
+        <v>129668.7</v>
+      </c>
+      <c r="F88" s="7">
+        <v>474854.7</v>
+      </c>
+      <c r="G88" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A89" s="5">
+        <v>87</v>
+      </c>
+      <c r="B89" s="7">
+        <v>129448</v>
+      </c>
+      <c r="C89" s="7">
+        <v>474946</v>
+      </c>
+      <c r="D89" s="7">
+        <v>232.8</v>
+      </c>
+      <c r="E89" s="7">
+        <v>129677.6</v>
+      </c>
+      <c r="F89" s="7">
+        <v>474907.2</v>
+      </c>
+      <c r="G89" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A90" s="5">
+        <v>88</v>
+      </c>
+      <c r="B90" s="7">
+        <v>129459</v>
+      </c>
+      <c r="C90" s="7">
+        <v>475021</v>
+      </c>
+      <c r="D90" s="7">
+        <v>234.5</v>
+      </c>
+      <c r="E90" s="7">
+        <v>129690.2</v>
+      </c>
+      <c r="F90" s="7">
+        <v>474982</v>
+      </c>
+      <c r="G90" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A91" s="5">
+        <v>89</v>
+      </c>
+      <c r="B91" s="7">
+        <v>129455</v>
+      </c>
+      <c r="C91" s="7">
+        <v>475091</v>
+      </c>
+      <c r="D91" s="7">
+        <v>250.1</v>
+      </c>
+      <c r="E91" s="7">
+        <v>129701.6</v>
+      </c>
+      <c r="F91" s="7">
+        <v>475049.4</v>
+      </c>
+      <c r="G91" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A92" s="5">
+        <v>90</v>
+      </c>
+      <c r="B92" s="7">
+        <v>129462</v>
+      </c>
+      <c r="C92" s="7">
+        <v>475175</v>
+      </c>
+      <c r="D92" s="7">
+        <v>257.2</v>
+      </c>
+      <c r="E92" s="7">
+        <v>129715.6</v>
+      </c>
+      <c r="F92" s="7">
+        <v>475132.2</v>
+      </c>
+      <c r="G92" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A93" s="5">
+        <v>91</v>
+      </c>
+      <c r="B93" s="7">
+        <v>129906</v>
+      </c>
+      <c r="C93" s="7">
+        <v>474702</v>
+      </c>
+      <c r="D93" s="7">
+        <v>259.39999999999998</v>
+      </c>
+      <c r="E93" s="7">
+        <v>129650.2</v>
+      </c>
+      <c r="F93" s="7">
+        <v>474745.2</v>
+      </c>
+      <c r="G93" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A94" s="5">
+        <v>92</v>
+      </c>
+      <c r="B94" s="7">
+        <v>129421</v>
+      </c>
+      <c r="C94" s="7">
+        <v>475158</v>
+      </c>
+      <c r="D94" s="7">
+        <v>294.7</v>
+      </c>
+      <c r="E94" s="7">
+        <v>129711.6</v>
+      </c>
+      <c r="F94" s="7">
+        <v>475108.9</v>
+      </c>
+      <c r="G94" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A95" s="5">
+        <v>93</v>
+      </c>
+      <c r="B95" s="7">
+        <v>129411</v>
+      </c>
+      <c r="C95" s="7">
+        <v>475134</v>
+      </c>
+      <c r="D95" s="7">
+        <v>300.60000000000002</v>
+      </c>
+      <c r="E95" s="7">
+        <v>129707.4</v>
+      </c>
+      <c r="F95" s="7">
+        <v>475083.9</v>
+      </c>
+      <c r="G95" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A96" s="5">
+        <v>94</v>
+      </c>
+      <c r="B96" s="7">
+        <v>130031</v>
+      </c>
+      <c r="C96" s="7">
+        <v>475178</v>
+      </c>
+      <c r="D96" s="7">
+        <v>303.39999999999998</v>
+      </c>
+      <c r="E96" s="7">
+        <v>129731.8</v>
+      </c>
+      <c r="F96" s="7">
+        <v>475228.5</v>
+      </c>
+      <c r="G96" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A97" s="5">
+        <v>95</v>
+      </c>
+      <c r="B97" s="7">
+        <v>128908</v>
+      </c>
+      <c r="C97" s="7">
+        <v>474710</v>
+      </c>
+      <c r="D97" s="7">
+        <v>725.3</v>
+      </c>
+      <c r="E97" s="7">
+        <v>129622.7</v>
+      </c>
+      <c r="F97" s="7">
+        <v>474586.2</v>
+      </c>
+      <c r="G97" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A98" s="5">
+        <v>96</v>
+      </c>
+      <c r="B98" s="7">
+        <v>128673</v>
+      </c>
+      <c r="C98" s="7">
+        <v>474700</v>
+      </c>
+      <c r="D98" s="7">
+        <v>955.2</v>
+      </c>
+      <c r="E98" s="7">
+        <v>129614.2</v>
+      </c>
+      <c r="F98" s="7">
+        <v>474537</v>
+      </c>
+      <c r="G98" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A99" s="5">
+        <v>97</v>
+      </c>
+      <c r="B99" s="7">
+        <v>129524</v>
+      </c>
+      <c r="C99" s="7">
+        <v>474445</v>
+      </c>
+      <c r="D99" s="7">
+        <v>73.099999999999994</v>
+      </c>
+      <c r="E99" s="7">
+        <v>129596.1</v>
+      </c>
+      <c r="F99" s="7">
+        <v>474432.5</v>
+      </c>
+      <c r="G99" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A100" s="5">
+        <v>98</v>
+      </c>
+      <c r="B100" s="7">
+        <v>129649</v>
+      </c>
+      <c r="C100" s="7">
+        <v>474217</v>
+      </c>
+      <c r="D100" s="7">
+        <v>88.9</v>
+      </c>
+      <c r="E100" s="7">
+        <v>129561.4</v>
+      </c>
+      <c r="F100" s="7">
+        <v>474232.2</v>
+      </c>
+      <c r="G100" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A101" s="5">
+        <v>99</v>
+      </c>
+      <c r="B101" s="7">
+        <v>129659</v>
+      </c>
+      <c r="C101" s="7">
+        <v>474153</v>
+      </c>
+      <c r="D101" s="7">
+        <v>109.7</v>
+      </c>
+      <c r="E101" s="7">
+        <v>129550.9</v>
+      </c>
+      <c r="F101" s="7">
+        <v>474171.7</v>
+      </c>
+      <c r="G101" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A102" s="5">
+        <v>100</v>
+      </c>
+      <c r="B102" s="7">
+        <v>129694</v>
+      </c>
+      <c r="C102" s="7">
+        <v>474235</v>
+      </c>
+      <c r="D102" s="7">
+        <v>130.19999999999999</v>
+      </c>
+      <c r="E102" s="7">
+        <v>129565.7</v>
+      </c>
+      <c r="F102" s="7">
+        <v>474257.2</v>
+      </c>
+      <c r="G102" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A103" s="5">
+        <v>101</v>
+      </c>
+      <c r="B103" s="7">
+        <v>129378</v>
+      </c>
+      <c r="C103" s="7">
+        <v>473986</v>
+      </c>
+      <c r="D103" s="7">
+        <v>138.69999999999999</v>
+      </c>
+      <c r="E103" s="7">
+        <v>129514.6</v>
+      </c>
+      <c r="F103" s="7">
+        <v>473962.3</v>
+      </c>
+      <c r="G103" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A104" s="5">
+        <v>102</v>
+      </c>
+      <c r="B104" s="7">
+        <v>129381</v>
+      </c>
+      <c r="C104" s="7">
+        <v>474016</v>
+      </c>
+      <c r="D104" s="7">
+        <v>140.80000000000001</v>
+      </c>
+      <c r="E104" s="7">
+        <v>129519.8</v>
+      </c>
+      <c r="F104" s="7">
+        <v>473992</v>
+      </c>
+      <c r="G104" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A105" s="5">
+        <v>103</v>
+      </c>
+      <c r="B105" s="7">
+        <v>129381</v>
+      </c>
+      <c r="C105" s="7">
+        <v>474055</v>
+      </c>
+      <c r="D105" s="7">
+        <v>147.5</v>
+      </c>
+      <c r="E105" s="7">
+        <v>129526.3</v>
+      </c>
+      <c r="F105" s="7">
+        <v>474029.8</v>
+      </c>
+      <c r="G105" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A106" s="5">
+        <v>104</v>
+      </c>
+      <c r="B106" s="7">
+        <v>129701</v>
+      </c>
+      <c r="C106" s="7">
+        <v>474153</v>
+      </c>
+      <c r="D106" s="7">
+        <v>151.1</v>
+      </c>
+      <c r="E106" s="7">
+        <v>129552.1</v>
+      </c>
+      <c r="F106" s="7">
+        <v>474178.8</v>
+      </c>
+      <c r="G106" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A107" s="5">
+        <v>105</v>
+      </c>
+      <c r="B107" s="7">
+        <v>129390</v>
+      </c>
+      <c r="C107" s="7">
+        <v>474155</v>
+      </c>
+      <c r="D107" s="7">
+        <v>155.69999999999999</v>
+      </c>
+      <c r="E107" s="7">
+        <v>129543.4</v>
+      </c>
+      <c r="F107" s="7">
+        <v>474128.4</v>
+      </c>
+      <c r="G107" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A108" s="5">
+        <v>106</v>
+      </c>
+      <c r="B108" s="7">
+        <v>129392</v>
+      </c>
+      <c r="C108" s="7">
+        <v>474232</v>
+      </c>
+      <c r="D108" s="7">
+        <v>166.9</v>
+      </c>
+      <c r="E108" s="7">
+        <v>129556.4</v>
+      </c>
+      <c r="F108" s="7">
+        <v>474203.5</v>
+      </c>
+      <c r="G108" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A109" s="5">
+        <v>107</v>
+      </c>
+      <c r="B109" s="7">
+        <v>129404</v>
+      </c>
+      <c r="C109" s="7">
+        <v>474332</v>
+      </c>
+      <c r="D109" s="7">
+        <v>172.1</v>
+      </c>
+      <c r="E109" s="7">
+        <v>129573.6</v>
+      </c>
+      <c r="F109" s="7">
+        <v>474302.6</v>
+      </c>
+      <c r="G109" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A110" s="5">
+        <v>108</v>
+      </c>
+      <c r="B110" s="7">
+        <v>129394</v>
+      </c>
+      <c r="C110" s="7">
+        <v>474284</v>
+      </c>
+      <c r="D110" s="7">
+        <v>173.8</v>
+      </c>
+      <c r="E110" s="7">
+        <v>129565.2</v>
+      </c>
+      <c r="F110" s="7">
+        <v>474254.4</v>
+      </c>
+      <c r="G110" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A111" s="5">
+        <v>109</v>
+      </c>
+      <c r="B111" s="7">
+        <v>129409</v>
+      </c>
+      <c r="C111" s="7">
+        <v>474376</v>
+      </c>
+      <c r="D111" s="7">
+        <v>174.7</v>
+      </c>
+      <c r="E111" s="7">
+        <v>129581.1</v>
+      </c>
+      <c r="F111" s="7">
+        <v>474346.2</v>
+      </c>
+      <c r="G111" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A112" s="5">
+        <v>110</v>
+      </c>
+      <c r="B112" s="7">
+        <v>129421</v>
+      </c>
+      <c r="C112" s="7">
+        <v>474463</v>
+      </c>
+      <c r="D112" s="7">
+        <v>177.7</v>
+      </c>
+      <c r="E112" s="7">
+        <v>129596.1</v>
+      </c>
+      <c r="F112" s="7">
+        <v>474432.7</v>
+      </c>
+      <c r="G112" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A113" s="5">
+        <v>111</v>
+      </c>
+      <c r="B113" s="7">
+        <v>129413</v>
+      </c>
+      <c r="C113" s="7">
+        <v>474427</v>
+      </c>
+      <c r="D113" s="7">
+        <v>179.4</v>
+      </c>
+      <c r="E113" s="7">
+        <v>129589.8</v>
+      </c>
+      <c r="F113" s="7">
+        <v>474396.4</v>
+      </c>
+      <c r="G113" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A114" s="5">
+        <v>112</v>
+      </c>
+      <c r="B114" s="7">
+        <v>129420</v>
+      </c>
+      <c r="C114" s="7">
+        <v>474502</v>
+      </c>
+      <c r="D114" s="7">
+        <v>185.3</v>
+      </c>
+      <c r="E114" s="7">
+        <v>129602.6</v>
+      </c>
+      <c r="F114" s="7">
+        <v>474470.40000000002</v>
+      </c>
+      <c r="G114" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A115" s="5">
+        <v>113</v>
+      </c>
+      <c r="B115" s="7">
+        <v>129754</v>
+      </c>
+      <c r="C115" s="7">
+        <v>474256</v>
+      </c>
+      <c r="D115" s="7">
+        <v>185.7</v>
+      </c>
+      <c r="E115" s="7">
+        <v>129571</v>
+      </c>
+      <c r="F115" s="7">
+        <v>474287.7</v>
+      </c>
+      <c r="G115" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A116" s="5">
+        <v>114</v>
+      </c>
+      <c r="B116" s="7">
+        <v>129820</v>
+      </c>
+      <c r="C116" s="7">
+        <v>474568</v>
+      </c>
+      <c r="D116" s="7">
+        <v>197.5</v>
+      </c>
+      <c r="E116" s="7">
+        <v>129625.4</v>
+      </c>
+      <c r="F116" s="7">
+        <v>474601.7</v>
+      </c>
+      <c r="G116" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A117" s="5">
+        <v>115</v>
+      </c>
+      <c r="B117" s="7">
+        <v>129759</v>
+      </c>
+      <c r="C117" s="7">
+        <v>474169</v>
+      </c>
+      <c r="D117" s="7">
+        <v>205.5</v>
+      </c>
+      <c r="E117" s="7">
+        <v>129556.5</v>
+      </c>
+      <c r="F117" s="7">
+        <v>474204.1</v>
+      </c>
+      <c r="G117" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A118" s="5">
+        <v>116</v>
+      </c>
+      <c r="B118" s="7">
+        <v>129857</v>
+      </c>
+      <c r="C118" s="7">
+        <v>474583</v>
+      </c>
+      <c r="D118" s="7">
+        <v>231.4</v>
+      </c>
+      <c r="E118" s="7">
+        <v>129629</v>
+      </c>
+      <c r="F118" s="7">
+        <v>474622.5</v>
+      </c>
+      <c r="G118" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A119" s="5">
+        <v>117</v>
+      </c>
+      <c r="B119" s="7">
+        <v>129845</v>
+      </c>
+      <c r="C119" s="7">
+        <v>474270</v>
+      </c>
+      <c r="D119" s="7">
+        <v>273</v>
+      </c>
+      <c r="E119" s="7">
+        <v>129576</v>
+      </c>
+      <c r="F119" s="7">
+        <v>474316.6</v>
+      </c>
+      <c r="G119" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A120" s="5">
+        <v>118</v>
+      </c>
+      <c r="B120" s="7">
+        <v>129837</v>
+      </c>
+      <c r="C120" s="7">
+        <v>474184</v>
+      </c>
+      <c r="D120" s="7">
+        <v>279.8</v>
+      </c>
+      <c r="E120" s="7">
+        <v>129561.3</v>
+      </c>
+      <c r="F120" s="7">
+        <v>474231.7</v>
+      </c>
+      <c r="G120" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A121" s="5">
+        <v>119</v>
+      </c>
+      <c r="B121" s="7">
+        <v>129857</v>
+      </c>
+      <c r="C121" s="7">
+        <v>474206</v>
+      </c>
+      <c r="D121" s="7">
+        <v>295.8</v>
+      </c>
+      <c r="E121" s="7">
+        <v>129565.6</v>
+      </c>
+      <c r="F121" s="7">
+        <v>474256.5</v>
+      </c>
+      <c r="G121" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A122" s="5">
+        <v>120</v>
+      </c>
+      <c r="B122" s="7">
+        <v>129895</v>
+      </c>
+      <c r="C122" s="7">
+        <v>474206</v>
+      </c>
+      <c r="D122" s="7">
+        <v>333.2</v>
+      </c>
+      <c r="E122" s="7">
+        <v>129566.7</v>
+      </c>
+      <c r="F122" s="7">
+        <v>474262.9</v>
+      </c>
+      <c r="G122" s="5">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G122">
+    <sortCondition ref="G2:G122"/>
+    <sortCondition ref="D2:D122"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C764B46-5E34-3D45-A366-6036CFA976BB}">
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>478867</v>
+      </c>
+      <c r="C2">
+        <v>478992</v>
+      </c>
+      <c r="D2">
+        <v>478163</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>477459</v>
+      </c>
+      <c r="C3">
+        <v>478163</v>
+      </c>
+      <c r="D3">
+        <v>476688.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>475918</v>
+      </c>
+      <c r="C4">
+        <v>476688.5</v>
+      </c>
+      <c r="D4">
+        <v>475642.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>475367</v>
+      </c>
+      <c r="C5">
+        <v>475642.5</v>
+      </c>
+      <c r="D5">
+        <v>475200</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>475033</v>
+      </c>
+      <c r="C6">
+        <v>475200</v>
+      </c>
+      <c r="D6">
+        <v>474588.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>474144</v>
+      </c>
+      <c r="C7">
+        <v>474588.5</v>
+      </c>
+      <c r="D7">
+        <v>473750.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>473357</v>
+      </c>
+      <c r="C8">
+        <v>473750.5</v>
+      </c>
+      <c r="D8">
+        <v>473105.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>472854</v>
+      </c>
+      <c r="C9">
+        <v>473105.5</v>
+      </c>
+      <c r="D9">
+        <v>472383</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>471912</v>
+      </c>
+      <c r="C10">
+        <v>472383</v>
+      </c>
+      <c r="D10">
+        <v>471028</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>470144</v>
+      </c>
+      <c r="C11">
+        <v>471028</v>
+      </c>
+      <c r="D11">
+        <v>469836</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>469528</v>
+      </c>
+      <c r="C12">
+        <v>469836</v>
+      </c>
+      <c r="D12">
+        <v>469043.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>468559</v>
+      </c>
+      <c r="C13">
+        <v>469043.5</v>
+      </c>
+      <c r="D13">
+        <v>467805.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>467052</v>
+      </c>
+      <c r="C14">
+        <v>467805.5</v>
+      </c>
+      <c r="D14">
+        <v>466927</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Analytische berekening toeveoeg. Bug met temperatuurverwerking uit het model gehaald. Weerstanden beschreven. ARK-temp statistieken berekend.
</commit_message>
<xml_diff>
--- a/Projects/ARK_RWS/images/peilbuizen/pb_tauw_XY.xlsx
+++ b/Projects/ARK_RWS/images/peilbuizen/pb_tauw_XY.xlsx
@@ -8,19 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Theo/Development/python/mf6_tools/mf6lab/Projects/ARK_RWS/images/peilbuizen/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6938CCB5-D9EA-8A46-B186-0ED956DBA414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBCAB357-67EC-8144-B7EE-87380E302C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1020" yWindow="1680" windowWidth="32360" windowHeight="20720" activeTab="1" xr2:uid="{E4383F88-647D-C347-BE79-FF24D0CA7E92}"/>
+    <workbookView xWindow="1020" yWindow="1680" windowWidth="32360" windowHeight="20720" xr2:uid="{E4383F88-647D-C347-BE79-FF24D0CA7E92}"/>
   </bookViews>
   <sheets>
     <sheet name="pbTauw" sheetId="1" r:id="rId1"/>
-    <sheet name="tempvariatie" sheetId="9" r:id="rId2"/>
-    <sheet name="pbKanaal" sheetId="3" r:id="rId3"/>
-    <sheet name="joined" sheetId="5" r:id="rId4"/>
-    <sheet name="Sheet2" sheetId="4" r:id="rId5"/>
-    <sheet name="laagopbouw" sheetId="6" r:id="rId6"/>
-    <sheet name="wellen" sheetId="7" r:id="rId7"/>
-    <sheet name="raaien" sheetId="8" r:id="rId8"/>
+    <sheet name="calibfation_raai6" sheetId="11" r:id="rId2"/>
+    <sheet name="tempvariatie" sheetId="9" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="10" r:id="rId4"/>
+    <sheet name="pbKanaal" sheetId="3" r:id="rId5"/>
+    <sheet name="joined" sheetId="5" r:id="rId6"/>
+    <sheet name="Sheet2" sheetId="4" r:id="rId7"/>
+    <sheet name="laagopbouw" sheetId="6" r:id="rId8"/>
+    <sheet name="wellen" sheetId="7" r:id="rId9"/>
+    <sheet name="raaien" sheetId="8" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="yyy" comment="Tijden en waarden van de stijghoogten gemiddeld over ca. 1 maand">Sheet2!$A$1:$G$67</definedName>
@@ -118,6 +120,73 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>tc={FECA8C00-68C0-DD46-B80A-61FAB26CD2FF}</author>
+    <author>tc={EA8B7049-F16D-1A4E-9B05-962D57FD7349}</author>
+    <author>tc={103F1F1E-1B0D-7A42-BA03-FE8C83672C88}</author>
+    <author>tc={B8FC59BC-7188-294B-A60F-B7A58596012C}</author>
+    <author>tc={E83EDFE8-9720-F742-949A-63A403E69D29}</author>
+    <author>tc={459752B2-D12C-D347-9E36-E91C0A2DE90F}</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{FECA8C00-68C0-DD46-B80A-61FAB26CD2FF}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    naam peilbuis</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="1" shapeId="0" xr:uid="{EA8B7049-F16D-1A4E-9B05-962D57FD7349}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    afstand (x,y) tot hartlijn ARK</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="2" shapeId="0" xr:uid="{103F1F1E-1B0D-7A42-BA03-FE8C83672C88}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    projectie van (x,y) op hartlijn ARK</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="3" shapeId="0" xr:uid="{B8FC59BC-7188-294B-A60F-B7A58596012C}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    projectie van (x,y) op hartlijn ARK</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="4" shapeId="0" xr:uid="{E83EDFE8-9720-F742-949A-63A403E69D29}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    https://experience.arcgis.com/experience/7a3706c6310e44d487de2e8b0888eac2
+Reply:
+    Vaak VP</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="5" shapeId="0" xr:uid="{459752B2-D12C-D347-9E36-E91C0A2DE90F}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Vastgestelde waterpeilen AGV
+Reply:
+    Vaak VP</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
     <author>tc={AC64C9D2-3F61-AF47-A662-FF8893F20A4A}</author>
   </authors>
   <commentList>
@@ -133,7 +202,7 @@
 </comments>
 </file>
 
-<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={EA54E30D-7CD8-1447-B295-5C3649868975}</author>
@@ -201,7 +270,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="148">
   <si>
     <t>x</t>
   </si>
@@ -583,16 +652,80 @@
   <si>
     <t>zijde v ARK</t>
   </si>
+  <si>
+    <t>cARK</t>
+  </si>
+  <si>
+    <t>Ra</t>
+  </si>
+  <si>
+    <t>phi_top_BX</t>
+  </si>
+  <si>
+    <t>q</t>
+  </si>
+  <si>
+    <t>Rb</t>
+  </si>
+  <si>
+    <t>phi_topBX</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>mm/d</t>
+  </si>
+  <si>
+    <t>dim</t>
+  </si>
+  <si>
+    <t>param</t>
+  </si>
+  <si>
+    <t>case 0</t>
+  </si>
+  <si>
+    <t>case 1</t>
+  </si>
+  <si>
+    <t>case 2</t>
+  </si>
+  <si>
+    <t>case 3</t>
+  </si>
+  <si>
+    <t>case 4</t>
+  </si>
+  <si>
+    <t>case 5</t>
+  </si>
+  <si>
+    <t>h_pold</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>h_ARK</t>
+  </si>
+  <si>
+    <t>phi_Bx-ddd</t>
+  </si>
+  <si>
+    <t>case 6</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -613,6 +746,40 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -622,7 +789,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -630,11 +797,128 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -646,8 +930,31 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1073,13 +1380,49 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="A1" dT="2026-06-01T22:36:03.63" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{FECA8C00-68C0-DD46-B80A-61FAB26CD2FF}">
+    <text>naam peilbuis</text>
+  </threadedComment>
+  <threadedComment ref="E1" dT="2026-06-01T22:35:37.02" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{EA8B7049-F16D-1A4E-9B05-962D57FD7349}">
+    <text>afstand (x,y) tot hartlijn ARK</text>
+  </threadedComment>
+  <threadedComment ref="F1" dT="2026-06-01T22:34:50.06" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{103F1F1E-1B0D-7A42-BA03-FE8C83672C88}">
+    <text>projectie van (x,y) op hartlijn ARK</text>
+  </threadedComment>
+  <threadedComment ref="G1" dT="2026-06-01T22:35:04.48" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{B8FC59BC-7188-294B-A60F-B7A58596012C}">
+    <text>projectie van (x,y) op hartlijn ARK</text>
+  </threadedComment>
+  <threadedComment ref="I1" dT="2026-06-02T11:32:50.06" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{E83EDFE8-9720-F742-949A-63A403E69D29}">
+    <text xml:space="preserve">https://experience.arcgis.com/experience/7a3706c6310e44d487de2e8b0888eac2
+</text>
+    <extLst>
+      <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
+        <xltc2:checksum>7762614</xltc2:checksum>
+        <xltc2:hyperlink startIndex="0" length="73" url="https://experience.arcgis.com/experience/7a3706c6310e44d487de2e8b0888eac2"/>
+      </x:ext>
+    </extLst>
+  </threadedComment>
+  <threadedComment ref="I1" dT="2026-06-02T11:33:52.99" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{BAF279BA-1480-DF4C-8547-4216DD59E977}" parentId="{E83EDFE8-9720-F742-949A-63A403E69D29}">
+    <text>Vaak VP</text>
+  </threadedComment>
+  <threadedComment ref="J1" dT="2026-06-02T11:33:15.19" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{459752B2-D12C-D347-9E36-E91C0A2DE90F}">
+    <text>Vastgestelde waterpeilen AGV</text>
+  </threadedComment>
+  <threadedComment ref="J1" dT="2026-06-02T11:33:36.77" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{76F57896-7048-F444-B8DF-DDDD046FAC38}" parentId="{459752B2-D12C-D347-9E36-E91C0A2DE90F}">
+    <text>Vaak VP</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment3.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="A1" dT="2026-06-02T15:10:45.11" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{AC64C9D2-3F61-AF47-A662-FF8893F20A4A}">
     <text>pb_sondering_in_en_naast_ARK</text>
   </threadedComment>
 </ThreadedComments>
 </file>
 
-<file path=xl/threadedComments/threadedComment3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/threadedComments/threadedComment4.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="A1" dT="2026-06-01T22:36:03.63" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{EA54E30D-7CD8-1447-B295-5C3649868975}">
     <text>naam peilbuis</text>
@@ -3592,7 +3935,7 @@
       <c r="I47">
         <v>-2.33</v>
       </c>
-      <c r="J47">
+      <c r="J47" s="29">
         <v>-2.33</v>
       </c>
       <c r="K47" t="str">
@@ -5277,7 +5620,424 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C764B46-5E34-3D45-A366-6036CFA976BB}">
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>478867</v>
+      </c>
+      <c r="C2">
+        <v>478992</v>
+      </c>
+      <c r="D2">
+        <v>478163</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>477459</v>
+      </c>
+      <c r="C3">
+        <v>478163</v>
+      </c>
+      <c r="D3">
+        <v>476688.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>475918</v>
+      </c>
+      <c r="C4">
+        <v>476688.5</v>
+      </c>
+      <c r="D4">
+        <v>475642.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>475367</v>
+      </c>
+      <c r="C5">
+        <v>475642.5</v>
+      </c>
+      <c r="D5">
+        <v>475200</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>475033</v>
+      </c>
+      <c r="C6">
+        <v>475200</v>
+      </c>
+      <c r="D6">
+        <v>474588.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>474144</v>
+      </c>
+      <c r="C7">
+        <v>474588.5</v>
+      </c>
+      <c r="D7">
+        <v>473750.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>473357</v>
+      </c>
+      <c r="C8">
+        <v>473750.5</v>
+      </c>
+      <c r="D8">
+        <v>473105.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>472854</v>
+      </c>
+      <c r="C9">
+        <v>473105.5</v>
+      </c>
+      <c r="D9">
+        <v>472383</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>471912</v>
+      </c>
+      <c r="C10">
+        <v>472383</v>
+      </c>
+      <c r="D10">
+        <v>471028</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>470144</v>
+      </c>
+      <c r="C11">
+        <v>471028</v>
+      </c>
+      <c r="D11">
+        <v>469836</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>469528</v>
+      </c>
+      <c r="C12">
+        <v>469836</v>
+      </c>
+      <c r="D12">
+        <v>469043.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>468559</v>
+      </c>
+      <c r="C13">
+        <v>469043.5</v>
+      </c>
+      <c r="D13">
+        <v>467805.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>467052</v>
+      </c>
+      <c r="C14">
+        <v>467805.5</v>
+      </c>
+      <c r="D14">
+        <v>466927</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A6B7A04-5F13-8A4E-9FE0-C5F28B59E7E3}">
+  <dimension ref="A1:P4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" t="s">
+        <v>8</v>
+      </c>
+      <c r="L1" t="s">
+        <v>86</v>
+      </c>
+      <c r="M1" t="s">
+        <v>85</v>
+      </c>
+      <c r="N1" t="s">
+        <v>84</v>
+      </c>
+      <c r="O1" t="s">
+        <v>89</v>
+      </c>
+      <c r="P1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A2" s="28">
+        <v>601</v>
+      </c>
+      <c r="B2" s="28">
+        <v>129045.2</v>
+      </c>
+      <c r="C2" s="28">
+        <v>474043.1</v>
+      </c>
+      <c r="D2" s="28">
+        <v>6</v>
+      </c>
+      <c r="E2" s="28">
+        <v>476.3</v>
+      </c>
+      <c r="F2" s="28">
+        <v>129515</v>
+      </c>
+      <c r="G2" s="28">
+        <v>473962</v>
+      </c>
+      <c r="H2" s="28">
+        <v>1</v>
+      </c>
+      <c r="I2" s="28">
+        <v>-2.6</v>
+      </c>
+      <c r="J2" s="28">
+        <v>-2.6</v>
+      </c>
+      <c r="K2" s="28" t="s">
+        <v>5</v>
+      </c>
+      <c r="L2" s="28">
+        <v>0</v>
+      </c>
+      <c r="M2" s="28">
+        <v>-1.5580000000000001</v>
+      </c>
+      <c r="N2" s="28">
+        <v>-1.698</v>
+      </c>
+      <c r="O2" s="28">
+        <v>-1.5580000000000001</v>
+      </c>
+      <c r="P2" s="28">
+        <v>-1.698</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A3" s="28">
+        <v>602</v>
+      </c>
+      <c r="B3" s="28">
+        <v>129311.3</v>
+      </c>
+      <c r="C3" s="28">
+        <v>474110.7</v>
+      </c>
+      <c r="D3" s="28">
+        <v>6</v>
+      </c>
+      <c r="E3" s="28">
+        <v>225.7</v>
+      </c>
+      <c r="F3" s="28">
+        <v>129534</v>
+      </c>
+      <c r="G3" s="28">
+        <v>474072</v>
+      </c>
+      <c r="H3" s="28">
+        <v>1</v>
+      </c>
+      <c r="I3" s="28">
+        <v>-2.6</v>
+      </c>
+      <c r="J3" s="28">
+        <v>-2.6</v>
+      </c>
+      <c r="K3" s="28" t="s">
+        <v>5</v>
+      </c>
+      <c r="L3" s="28">
+        <v>0</v>
+      </c>
+      <c r="M3" s="28">
+        <v>-1.415</v>
+      </c>
+      <c r="N3" s="28">
+        <v>-1.6359999999999999</v>
+      </c>
+      <c r="O3" s="28">
+        <v>-1.415</v>
+      </c>
+      <c r="P3" s="28">
+        <v>-1.6359999999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A4" s="28">
+        <v>603</v>
+      </c>
+      <c r="B4" s="28">
+        <v>129485.6</v>
+      </c>
+      <c r="C4" s="28">
+        <v>474227.9</v>
+      </c>
+      <c r="D4" s="28">
+        <v>6</v>
+      </c>
+      <c r="E4" s="28">
+        <v>73.900000000000006</v>
+      </c>
+      <c r="F4" s="28">
+        <v>129558</v>
+      </c>
+      <c r="G4" s="28">
+        <v>474215</v>
+      </c>
+      <c r="H4" s="28">
+        <v>1</v>
+      </c>
+      <c r="I4" s="28">
+        <v>-2.6</v>
+      </c>
+      <c r="J4" s="28">
+        <v>-2.6</v>
+      </c>
+      <c r="K4" s="28" t="s">
+        <v>5</v>
+      </c>
+      <c r="L4" s="28">
+        <v>0</v>
+      </c>
+      <c r="M4" s="28">
+        <v>-1.196</v>
+      </c>
+      <c r="N4" s="28">
+        <v>-1.4850000000000001</v>
+      </c>
+      <c r="O4" s="28">
+        <v>-1.196</v>
+      </c>
+      <c r="P4" s="28">
+        <v>-1.4850000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B88294E-026C-7C43-944B-85AEB4D9DBE0}">
   <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -5437,7 +6197,322 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DD048BC-F0C9-E948-9AD7-CE95095093FB}">
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="5" max="6" width="10.83203125" style="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B1" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="F1" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="G1" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="H1" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="I1" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="J1" s="14" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B2" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="C2" s="24" t="s">
+        <v>133</v>
+      </c>
+      <c r="D2" s="24">
+        <v>1E-3</v>
+      </c>
+      <c r="E2" s="24">
+        <v>1</v>
+      </c>
+      <c r="F2" s="24">
+        <v>5</v>
+      </c>
+      <c r="G2" s="24">
+        <v>10</v>
+      </c>
+      <c r="H2" s="24">
+        <v>17</v>
+      </c>
+      <c r="I2" s="24">
+        <v>20.5</v>
+      </c>
+      <c r="J2" s="25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B3" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="D3" s="16">
+        <v>-0.4</v>
+      </c>
+      <c r="E3" s="16">
+        <v>-0.4</v>
+      </c>
+      <c r="F3" s="16">
+        <v>-0.4</v>
+      </c>
+      <c r="G3" s="16">
+        <v>-0.4</v>
+      </c>
+      <c r="H3" s="16">
+        <v>-0.4</v>
+      </c>
+      <c r="I3" s="16"/>
+      <c r="J3" s="17">
+        <v>-0.4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>134</v>
+      </c>
+      <c r="D4" s="26">
+        <v>-0.65500000000000003</v>
+      </c>
+      <c r="E4" s="26">
+        <v>-0.7</v>
+      </c>
+      <c r="F4" s="26">
+        <v>-0.83799999999999997</v>
+      </c>
+      <c r="G4" s="26">
+        <v>-0.97499999999999998</v>
+      </c>
+      <c r="H4" s="26">
+        <v>-1.1259999999999999</v>
+      </c>
+      <c r="I4" s="26"/>
+      <c r="J4" s="27">
+        <v>-1.391</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B5" s="20" t="s">
+        <v>143</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="D5" s="21">
+        <v>-2.2999999999999998</v>
+      </c>
+      <c r="E5" s="21">
+        <v>-2.2999999999999998</v>
+      </c>
+      <c r="F5" s="21">
+        <v>-2.2999999999999998</v>
+      </c>
+      <c r="G5" s="21">
+        <v>-2.2999999999999998</v>
+      </c>
+      <c r="H5" s="21">
+        <v>-2.2999999999999998</v>
+      </c>
+      <c r="I5" s="21"/>
+      <c r="J5" s="22">
+        <v>-2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>131</v>
+      </c>
+      <c r="B6" s="23" t="s">
+        <v>130</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="D6" s="24">
+        <v>36.6</v>
+      </c>
+      <c r="E6" s="24">
+        <v>36.6</v>
+      </c>
+      <c r="F6" s="24">
+        <v>36.6</v>
+      </c>
+      <c r="G6" s="24">
+        <v>36.6</v>
+      </c>
+      <c r="H6" s="24">
+        <v>36.6</v>
+      </c>
+      <c r="I6" s="24"/>
+      <c r="J6" s="25">
+        <v>36.6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>128</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="D7" s="16">
+        <v>10.8</v>
+      </c>
+      <c r="E7" s="16">
+        <v>12.6</v>
+      </c>
+      <c r="F7" s="16">
+        <v>18.5</v>
+      </c>
+      <c r="G7" s="16">
+        <v>24.3</v>
+      </c>
+      <c r="H7" s="16">
+        <v>30.6</v>
+      </c>
+      <c r="I7" s="16"/>
+      <c r="J7" s="17">
+        <v>41.8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>130</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>131</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="D8" s="21">
+        <v>42.6</v>
+      </c>
+      <c r="E8" s="21">
+        <v>41.5</v>
+      </c>
+      <c r="F8" s="21">
+        <v>38</v>
+      </c>
+      <c r="G8" s="21">
+        <v>34.5</v>
+      </c>
+      <c r="H8" s="21">
+        <v>30.6</v>
+      </c>
+      <c r="I8" s="21"/>
+      <c r="J8" s="22">
+        <v>23.7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
+        <v>146</v>
+      </c>
+      <c r="D10" s="11">
+        <f>D4-$J$4</f>
+        <v>0.73599999999999999</v>
+      </c>
+      <c r="E10" s="11">
+        <f t="shared" ref="E10:J10" si="0">E4-$J$4</f>
+        <v>0.69100000000000006</v>
+      </c>
+      <c r="F10" s="11">
+        <f t="shared" si="0"/>
+        <v>0.55300000000000005</v>
+      </c>
+      <c r="G10" s="11">
+        <f t="shared" si="0"/>
+        <v>0.41600000000000004</v>
+      </c>
+      <c r="H10" s="11">
+        <f t="shared" si="0"/>
+        <v>0.26500000000000012</v>
+      </c>
+      <c r="I10" s="11"/>
+      <c r="J10" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E12" s="12">
+        <f>35/1.7</f>
+        <v>20.588235294117649</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E13" s="12">
+        <f>10.5/1.7</f>
+        <v>6.1764705882352944</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E14" s="12">
+        <f>41.8/1.7</f>
+        <v>24.588235294117645</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B16">
+        <v>5</v>
+      </c>
+      <c r="C16">
+        <f>30/(20+B16)</f>
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B17">
+        <v>25</v>
+      </c>
+      <c r="C17">
+        <f>30/(20+B17)</f>
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C2120DA-4889-CE46-967A-1E97B2CF047D}">
   <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -6001,7 +7076,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E4B153B-BE8A-8445-8BB9-AE4D4CAEE74C}">
   <dimension ref="A1:O88"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -10148,7 +11223,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55E721B4-ED8E-434B-9DEE-2C2B14F64426}">
   <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -11465,7 +12540,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BE2EFF2-13EC-F842-8DF0-C6F8E64FF8D5}">
   <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -11686,7 +12761,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7C0FFF9-DB26-954D-871D-A338BC7B0C37}">
   <dimension ref="A1:G122"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -14507,210 +15582,4 @@
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C764B46-5E34-3D45-A366-6036CFA976BB}">
-  <dimension ref="A1:D14"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>478867</v>
-      </c>
-      <c r="C2">
-        <v>478992</v>
-      </c>
-      <c r="D2">
-        <v>478163</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>477459</v>
-      </c>
-      <c r="C3">
-        <v>478163</v>
-      </c>
-      <c r="D3">
-        <v>476688.5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>475918</v>
-      </c>
-      <c r="C4">
-        <v>476688.5</v>
-      </c>
-      <c r="D4">
-        <v>475642.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>475367</v>
-      </c>
-      <c r="C5">
-        <v>475642.5</v>
-      </c>
-      <c r="D5">
-        <v>475200</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>475033</v>
-      </c>
-      <c r="C6">
-        <v>475200</v>
-      </c>
-      <c r="D6">
-        <v>474588.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>474144</v>
-      </c>
-      <c r="C7">
-        <v>474588.5</v>
-      </c>
-      <c r="D7">
-        <v>473750.5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>473357</v>
-      </c>
-      <c r="C8">
-        <v>473750.5</v>
-      </c>
-      <c r="D8">
-        <v>473105.5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9">
-        <v>472854</v>
-      </c>
-      <c r="C9">
-        <v>473105.5</v>
-      </c>
-      <c r="D9">
-        <v>472383</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10">
-        <v>471912</v>
-      </c>
-      <c r="C10">
-        <v>472383</v>
-      </c>
-      <c r="D10">
-        <v>471028</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11">
-        <v>470144</v>
-      </c>
-      <c r="C11">
-        <v>471028</v>
-      </c>
-      <c r="D11">
-        <v>469836</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12">
-        <v>469528</v>
-      </c>
-      <c r="C12">
-        <v>469836</v>
-      </c>
-      <c r="D12">
-        <v>469043.5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13">
-        <v>468559</v>
-      </c>
-      <c r="C13">
-        <v>469043.5</v>
-      </c>
-      <c r="D13">
-        <v>467805.5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14">
-        <v>467052</v>
-      </c>
-      <c r="C14">
-        <v>467805.5</v>
-      </c>
-      <c r="D14">
-        <v>466927</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Almost ready. Text nog afronden.
</commit_message>
<xml_diff>
--- a/Projects/ARK_RWS/images/peilbuizen/pb_tauw_XY.xlsx
+++ b/Projects/ARK_RWS/images/peilbuizen/pb_tauw_XY.xlsx
@@ -8,21 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Theo/Development/python/mf6_tools/mf6lab/Projects/ARK_RWS/images/peilbuizen/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBCAB357-67EC-8144-B7EE-87380E302C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F148F20-8D91-4D40-BDF1-2E6726A06293}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1020" yWindow="1680" windowWidth="32360" windowHeight="20720" xr2:uid="{E4383F88-647D-C347-BE79-FF24D0CA7E92}"/>
+    <workbookView xWindow="-1140" yWindow="-21520" windowWidth="32360" windowHeight="20720" activeTab="1" xr2:uid="{E4383F88-647D-C347-BE79-FF24D0CA7E92}"/>
   </bookViews>
   <sheets>
     <sheet name="pbTauw" sheetId="1" r:id="rId1"/>
-    <sheet name="calibfation_raai6" sheetId="11" r:id="rId2"/>
-    <sheet name="tempvariatie" sheetId="9" r:id="rId3"/>
-    <sheet name="Sheet1" sheetId="10" r:id="rId4"/>
-    <sheet name="pbKanaal" sheetId="3" r:id="rId5"/>
-    <sheet name="joined" sheetId="5" r:id="rId6"/>
-    <sheet name="Sheet2" sheetId="4" r:id="rId7"/>
-    <sheet name="laagopbouw" sheetId="6" r:id="rId8"/>
-    <sheet name="wellen" sheetId="7" r:id="rId9"/>
-    <sheet name="raaien" sheetId="8" r:id="rId10"/>
+    <sheet name="Sheet1" sheetId="10" r:id="rId2"/>
+    <sheet name="pbKanaal" sheetId="3" r:id="rId3"/>
+    <sheet name="joined" sheetId="5" r:id="rId4"/>
+    <sheet name="Sheet2" sheetId="4" r:id="rId5"/>
+    <sheet name="laagopbouw" sheetId="6" r:id="rId6"/>
+    <sheet name="wellen" sheetId="7" r:id="rId7"/>
+    <sheet name="raaien" sheetId="8" r:id="rId8"/>
+    <sheet name="calibfation_raai6" sheetId="11" r:id="rId9"/>
+    <sheet name="tempvariatie" sheetId="9" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="yyy" comment="Tijden en waarden van de stijghoogten gemiddeld over ca. 1 maand">Sheet2!$A$1:$G$67</definedName>
@@ -120,73 +120,6 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={FECA8C00-68C0-DD46-B80A-61FAB26CD2FF}</author>
-    <author>tc={EA8B7049-F16D-1A4E-9B05-962D57FD7349}</author>
-    <author>tc={103F1F1E-1B0D-7A42-BA03-FE8C83672C88}</author>
-    <author>tc={B8FC59BC-7188-294B-A60F-B7A58596012C}</author>
-    <author>tc={E83EDFE8-9720-F742-949A-63A403E69D29}</author>
-    <author>tc={459752B2-D12C-D347-9E36-E91C0A2DE90F}</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{FECA8C00-68C0-DD46-B80A-61FAB26CD2FF}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    naam peilbuis</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="1" shapeId="0" xr:uid="{EA8B7049-F16D-1A4E-9B05-962D57FD7349}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    afstand (x,y) tot hartlijn ARK</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="2" shapeId="0" xr:uid="{103F1F1E-1B0D-7A42-BA03-FE8C83672C88}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    projectie van (x,y) op hartlijn ARK</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="3" shapeId="0" xr:uid="{B8FC59BC-7188-294B-A60F-B7A58596012C}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    projectie van (x,y) op hartlijn ARK</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="4" shapeId="0" xr:uid="{E83EDFE8-9720-F742-949A-63A403E69D29}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    https://experience.arcgis.com/experience/7a3706c6310e44d487de2e8b0888eac2
-Reply:
-    Vaak VP</t>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="5" shapeId="0" xr:uid="{459752B2-D12C-D347-9E36-E91C0A2DE90F}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Vastgestelde waterpeilen AGV
-Reply:
-    Vaak VP</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
     <author>tc={AC64C9D2-3F61-AF47-A662-FF8893F20A4A}</author>
   </authors>
   <commentList>
@@ -202,7 +135,7 @@
 </comments>
 </file>
 
-<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={EA54E30D-7CD8-1447-B295-5C3649868975}</author>
@@ -269,8 +202,75 @@
 </comments>
 </file>
 
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={FECA8C00-68C0-DD46-B80A-61FAB26CD2FF}</author>
+    <author>tc={EA8B7049-F16D-1A4E-9B05-962D57FD7349}</author>
+    <author>tc={103F1F1E-1B0D-7A42-BA03-FE8C83672C88}</author>
+    <author>tc={B8FC59BC-7188-294B-A60F-B7A58596012C}</author>
+    <author>tc={E83EDFE8-9720-F742-949A-63A403E69D29}</author>
+    <author>tc={459752B2-D12C-D347-9E36-E91C0A2DE90F}</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{FECA8C00-68C0-DD46-B80A-61FAB26CD2FF}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    naam peilbuis</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="1" shapeId="0" xr:uid="{EA8B7049-F16D-1A4E-9B05-962D57FD7349}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    afstand (x,y) tot hartlijn ARK</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="2" shapeId="0" xr:uid="{103F1F1E-1B0D-7A42-BA03-FE8C83672C88}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    projectie van (x,y) op hartlijn ARK</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="3" shapeId="0" xr:uid="{B8FC59BC-7188-294B-A60F-B7A58596012C}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    projectie van (x,y) op hartlijn ARK</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="4" shapeId="0" xr:uid="{E83EDFE8-9720-F742-949A-63A403E69D29}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    https://experience.arcgis.com/experience/7a3706c6310e44d487de2e8b0888eac2
+Reply:
+    Vaak VP</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="5" shapeId="0" xr:uid="{459752B2-D12C-D347-9E36-E91C0A2DE90F}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Vastgestelde waterpeilen AGV
+Reply:
+    Vaak VP</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="158">
   <si>
     <t>x</t>
   </si>
@@ -715,6 +715,36 @@
   <si>
     <t>case 6</t>
   </si>
+  <si>
+    <t>seizoen</t>
+  </si>
+  <si>
+    <t>temp ARK</t>
+  </si>
+  <si>
+    <t>c_ARK</t>
+  </si>
+  <si>
+    <t>q_inf</t>
+  </si>
+  <si>
+    <t>hBX_bot</t>
+  </si>
+  <si>
+    <t>analytisch</t>
+  </si>
+  <si>
+    <t>zomer</t>
+  </si>
+  <si>
+    <t>q_z/q_w</t>
+  </si>
+  <si>
+    <t>dhZ/dhW</t>
+  </si>
+  <si>
+    <t>ARK temp (2024, 2025)</t>
+  </si>
 </sst>
 </file>
 
@@ -725,7 +755,7 @@
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -767,12 +797,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
       <u/>
       <sz val="12"/>
       <color theme="1"/>
@@ -781,12 +805,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="12">
@@ -918,7 +948,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -944,17 +974,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1380,49 +1413,13 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A1" dT="2026-06-01T22:36:03.63" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{FECA8C00-68C0-DD46-B80A-61FAB26CD2FF}">
-    <text>naam peilbuis</text>
-  </threadedComment>
-  <threadedComment ref="E1" dT="2026-06-01T22:35:37.02" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{EA8B7049-F16D-1A4E-9B05-962D57FD7349}">
-    <text>afstand (x,y) tot hartlijn ARK</text>
-  </threadedComment>
-  <threadedComment ref="F1" dT="2026-06-01T22:34:50.06" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{103F1F1E-1B0D-7A42-BA03-FE8C83672C88}">
-    <text>projectie van (x,y) op hartlijn ARK</text>
-  </threadedComment>
-  <threadedComment ref="G1" dT="2026-06-01T22:35:04.48" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{B8FC59BC-7188-294B-A60F-B7A58596012C}">
-    <text>projectie van (x,y) op hartlijn ARK</text>
-  </threadedComment>
-  <threadedComment ref="I1" dT="2026-06-02T11:32:50.06" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{E83EDFE8-9720-F742-949A-63A403E69D29}">
-    <text xml:space="preserve">https://experience.arcgis.com/experience/7a3706c6310e44d487de2e8b0888eac2
-</text>
-    <extLst>
-      <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
-        <xltc2:checksum>7762614</xltc2:checksum>
-        <xltc2:hyperlink startIndex="0" length="73" url="https://experience.arcgis.com/experience/7a3706c6310e44d487de2e8b0888eac2"/>
-      </x:ext>
-    </extLst>
-  </threadedComment>
-  <threadedComment ref="I1" dT="2026-06-02T11:33:52.99" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{BAF279BA-1480-DF4C-8547-4216DD59E977}" parentId="{E83EDFE8-9720-F742-949A-63A403E69D29}">
-    <text>Vaak VP</text>
-  </threadedComment>
-  <threadedComment ref="J1" dT="2026-06-02T11:33:15.19" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{459752B2-D12C-D347-9E36-E91C0A2DE90F}">
-    <text>Vastgestelde waterpeilen AGV</text>
-  </threadedComment>
-  <threadedComment ref="J1" dT="2026-06-02T11:33:36.77" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{76F57896-7048-F444-B8DF-DDDD046FAC38}" parentId="{459752B2-D12C-D347-9E36-E91C0A2DE90F}">
-    <text>Vaak VP</text>
-  </threadedComment>
-</ThreadedComments>
-</file>
-
-<file path=xl/threadedComments/threadedComment3.xml><?xml version="1.0" encoding="utf-8"?>
-<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="A1" dT="2026-06-02T15:10:45.11" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{AC64C9D2-3F61-AF47-A662-FF8893F20A4A}">
     <text>pb_sondering_in_en_naast_ARK</text>
   </threadedComment>
 </ThreadedComments>
 </file>
 
-<file path=xl/threadedComments/threadedComment4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/threadedComments/threadedComment3.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="A1" dT="2026-06-01T22:36:03.63" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{EA54E30D-7CD8-1447-B295-5C3649868975}">
     <text>naam peilbuis</text>
@@ -1458,6 +1455,42 @@
 </ThreadedComments>
 </file>
 
+<file path=xl/threadedComments/threadedComment4.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="A1" dT="2026-06-01T22:36:03.63" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{FECA8C00-68C0-DD46-B80A-61FAB26CD2FF}">
+    <text>naam peilbuis</text>
+  </threadedComment>
+  <threadedComment ref="E1" dT="2026-06-01T22:35:37.02" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{EA8B7049-F16D-1A4E-9B05-962D57FD7349}">
+    <text>afstand (x,y) tot hartlijn ARK</text>
+  </threadedComment>
+  <threadedComment ref="F1" dT="2026-06-01T22:34:50.06" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{103F1F1E-1B0D-7A42-BA03-FE8C83672C88}">
+    <text>projectie van (x,y) op hartlijn ARK</text>
+  </threadedComment>
+  <threadedComment ref="G1" dT="2026-06-01T22:35:04.48" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{B8FC59BC-7188-294B-A60F-B7A58596012C}">
+    <text>projectie van (x,y) op hartlijn ARK</text>
+  </threadedComment>
+  <threadedComment ref="I1" dT="2026-06-02T11:32:50.06" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{E83EDFE8-9720-F742-949A-63A403E69D29}">
+    <text xml:space="preserve">https://experience.arcgis.com/experience/7a3706c6310e44d487de2e8b0888eac2
+</text>
+    <extLst>
+      <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
+        <xltc2:checksum>7762614</xltc2:checksum>
+        <xltc2:hyperlink startIndex="0" length="73" url="https://experience.arcgis.com/experience/7a3706c6310e44d487de2e8b0888eac2"/>
+      </x:ext>
+    </extLst>
+  </threadedComment>
+  <threadedComment ref="I1" dT="2026-06-02T11:33:52.99" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{BAF279BA-1480-DF4C-8547-4216DD59E977}" parentId="{E83EDFE8-9720-F742-949A-63A403E69D29}">
+    <text>Vaak VP</text>
+  </threadedComment>
+  <threadedComment ref="J1" dT="2026-06-02T11:33:15.19" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{459752B2-D12C-D347-9E36-E91C0A2DE90F}">
+    <text>Vastgestelde waterpeilen AGV</text>
+  </threadedComment>
+  <threadedComment ref="J1" dT="2026-06-02T11:33:36.77" personId="{96A1243A-EDAC-3347-8C18-15E2B014F1F1}" id="{76F57896-7048-F444-B8DF-DDDD046FAC38}" parentId="{459752B2-D12C-D347-9E36-E91C0A2DE90F}">
+    <text>Vaak VP</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9242C9A1-0ECC-C140-AC02-EB1C99BC61A4}">
   <dimension ref="A1:P78"/>
@@ -3935,7 +3968,7 @@
       <c r="I47">
         <v>-2.33</v>
       </c>
-      <c r="J47" s="29">
+      <c r="J47" s="27">
         <v>-2.33</v>
       </c>
       <c r="K47" t="str">
@@ -5621,423 +5654,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C764B46-5E34-3D45-A366-6036CFA976BB}">
-  <dimension ref="A1:D14"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>478867</v>
-      </c>
-      <c r="C2">
-        <v>478992</v>
-      </c>
-      <c r="D2">
-        <v>478163</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>477459</v>
-      </c>
-      <c r="C3">
-        <v>478163</v>
-      </c>
-      <c r="D3">
-        <v>476688.5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>475918</v>
-      </c>
-      <c r="C4">
-        <v>476688.5</v>
-      </c>
-      <c r="D4">
-        <v>475642.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>475367</v>
-      </c>
-      <c r="C5">
-        <v>475642.5</v>
-      </c>
-      <c r="D5">
-        <v>475200</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>475033</v>
-      </c>
-      <c r="C6">
-        <v>475200</v>
-      </c>
-      <c r="D6">
-        <v>474588.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>474144</v>
-      </c>
-      <c r="C7">
-        <v>474588.5</v>
-      </c>
-      <c r="D7">
-        <v>473750.5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>473357</v>
-      </c>
-      <c r="C8">
-        <v>473750.5</v>
-      </c>
-      <c r="D8">
-        <v>473105.5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9">
-        <v>472854</v>
-      </c>
-      <c r="C9">
-        <v>473105.5</v>
-      </c>
-      <c r="D9">
-        <v>472383</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10">
-        <v>471912</v>
-      </c>
-      <c r="C10">
-        <v>472383</v>
-      </c>
-      <c r="D10">
-        <v>471028</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11">
-        <v>470144</v>
-      </c>
-      <c r="C11">
-        <v>471028</v>
-      </c>
-      <c r="D11">
-        <v>469836</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12">
-        <v>469528</v>
-      </c>
-      <c r="C12">
-        <v>469836</v>
-      </c>
-      <c r="D12">
-        <v>469043.5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13">
-        <v>468559</v>
-      </c>
-      <c r="C13">
-        <v>469043.5</v>
-      </c>
-      <c r="D13">
-        <v>467805.5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14">
-        <v>467052</v>
-      </c>
-      <c r="C14">
-        <v>467805.5</v>
-      </c>
-      <c r="D14">
-        <v>466927</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A6B7A04-5F13-8A4E-9FE0-C5F28B59E7E3}">
-  <dimension ref="A1:P4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1" t="s">
-        <v>6</v>
-      </c>
-      <c r="J1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" t="s">
-        <v>8</v>
-      </c>
-      <c r="L1" t="s">
-        <v>86</v>
-      </c>
-      <c r="M1" t="s">
-        <v>85</v>
-      </c>
-      <c r="N1" t="s">
-        <v>84</v>
-      </c>
-      <c r="O1" t="s">
-        <v>89</v>
-      </c>
-      <c r="P1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A2" s="28">
-        <v>601</v>
-      </c>
-      <c r="B2" s="28">
-        <v>129045.2</v>
-      </c>
-      <c r="C2" s="28">
-        <v>474043.1</v>
-      </c>
-      <c r="D2" s="28">
-        <v>6</v>
-      </c>
-      <c r="E2" s="28">
-        <v>476.3</v>
-      </c>
-      <c r="F2" s="28">
-        <v>129515</v>
-      </c>
-      <c r="G2" s="28">
-        <v>473962</v>
-      </c>
-      <c r="H2" s="28">
-        <v>1</v>
-      </c>
-      <c r="I2" s="28">
-        <v>-2.6</v>
-      </c>
-      <c r="J2" s="28">
-        <v>-2.6</v>
-      </c>
-      <c r="K2" s="28" t="s">
-        <v>5</v>
-      </c>
-      <c r="L2" s="28">
-        <v>0</v>
-      </c>
-      <c r="M2" s="28">
-        <v>-1.5580000000000001</v>
-      </c>
-      <c r="N2" s="28">
-        <v>-1.698</v>
-      </c>
-      <c r="O2" s="28">
-        <v>-1.5580000000000001</v>
-      </c>
-      <c r="P2" s="28">
-        <v>-1.698</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A3" s="28">
-        <v>602</v>
-      </c>
-      <c r="B3" s="28">
-        <v>129311.3</v>
-      </c>
-      <c r="C3" s="28">
-        <v>474110.7</v>
-      </c>
-      <c r="D3" s="28">
-        <v>6</v>
-      </c>
-      <c r="E3" s="28">
-        <v>225.7</v>
-      </c>
-      <c r="F3" s="28">
-        <v>129534</v>
-      </c>
-      <c r="G3" s="28">
-        <v>474072</v>
-      </c>
-      <c r="H3" s="28">
-        <v>1</v>
-      </c>
-      <c r="I3" s="28">
-        <v>-2.6</v>
-      </c>
-      <c r="J3" s="28">
-        <v>-2.6</v>
-      </c>
-      <c r="K3" s="28" t="s">
-        <v>5</v>
-      </c>
-      <c r="L3" s="28">
-        <v>0</v>
-      </c>
-      <c r="M3" s="28">
-        <v>-1.415</v>
-      </c>
-      <c r="N3" s="28">
-        <v>-1.6359999999999999</v>
-      </c>
-      <c r="O3" s="28">
-        <v>-1.415</v>
-      </c>
-      <c r="P3" s="28">
-        <v>-1.6359999999999999</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A4" s="28">
-        <v>603</v>
-      </c>
-      <c r="B4" s="28">
-        <v>129485.6</v>
-      </c>
-      <c r="C4" s="28">
-        <v>474227.9</v>
-      </c>
-      <c r="D4" s="28">
-        <v>6</v>
-      </c>
-      <c r="E4" s="28">
-        <v>73.900000000000006</v>
-      </c>
-      <c r="F4" s="28">
-        <v>129558</v>
-      </c>
-      <c r="G4" s="28">
-        <v>474215</v>
-      </c>
-      <c r="H4" s="28">
-        <v>1</v>
-      </c>
-      <c r="I4" s="28">
-        <v>-2.6</v>
-      </c>
-      <c r="J4" s="28">
-        <v>-2.6</v>
-      </c>
-      <c r="K4" s="28" t="s">
-        <v>5</v>
-      </c>
-      <c r="L4" s="28">
-        <v>0</v>
-      </c>
-      <c r="M4" s="28">
-        <v>-1.196</v>
-      </c>
-      <c r="N4" s="28">
-        <v>-1.4850000000000001</v>
-      </c>
-      <c r="O4" s="28">
-        <v>-1.196</v>
-      </c>
-      <c r="P4" s="28">
-        <v>-1.4850000000000001</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B88294E-026C-7C43-944B-85AEB4D9DBE0}">
   <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -6197,12 +5813,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DD048BC-F0C9-E948-9AD7-CE95095093FB}">
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="6" width="10.83203125" style="12"/>
+    <col min="8" max="8" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
@@ -6238,31 +5855,31 @@
       <c r="A2" t="s">
         <v>127</v>
       </c>
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="23" t="s">
         <v>133</v>
       </c>
-      <c r="D2" s="24">
+      <c r="D2" s="23">
         <v>1E-3</v>
       </c>
-      <c r="E2" s="24">
+      <c r="E2" s="23">
         <v>1</v>
       </c>
-      <c r="F2" s="24">
+      <c r="F2" s="23">
         <v>5</v>
       </c>
-      <c r="G2" s="24">
+      <c r="G2" s="23">
         <v>10</v>
       </c>
-      <c r="H2" s="24">
+      <c r="H2" s="23">
         <v>17</v>
       </c>
-      <c r="I2" s="24">
+      <c r="I2" s="23">
         <v>20.5</v>
       </c>
-      <c r="J2" s="25">
+      <c r="J2" s="24">
         <v>35</v>
       </c>
     </row>
@@ -6300,53 +5917,53 @@
       <c r="B4" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" t="s">
         <v>134</v>
       </c>
-      <c r="D4" s="26">
+      <c r="D4" s="11">
         <v>-0.65500000000000003</v>
       </c>
-      <c r="E4" s="26">
+      <c r="E4" s="11">
         <v>-0.7</v>
       </c>
-      <c r="F4" s="26">
+      <c r="F4" s="11">
         <v>-0.83799999999999997</v>
       </c>
-      <c r="G4" s="26">
+      <c r="G4" s="11">
         <v>-0.97499999999999998</v>
       </c>
-      <c r="H4" s="26">
+      <c r="H4" s="11">
         <v>-1.1259999999999999</v>
       </c>
-      <c r="I4" s="26"/>
-      <c r="J4" s="27">
+      <c r="I4" s="11"/>
+      <c r="J4" s="25">
         <v>-1.391</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="20" t="s">
         <v>144</v>
       </c>
-      <c r="D5" s="21">
+      <c r="D5" s="20">
         <v>-2.2999999999999998</v>
       </c>
-      <c r="E5" s="21">
+      <c r="E5" s="20">
         <v>-2.2999999999999998</v>
       </c>
-      <c r="F5" s="21">
+      <c r="F5" s="20">
         <v>-2.2999999999999998</v>
       </c>
-      <c r="G5" s="21">
+      <c r="G5" s="20">
         <v>-2.2999999999999998</v>
       </c>
-      <c r="H5" s="21">
+      <c r="H5" s="20">
         <v>-2.2999999999999998</v>
       </c>
-      <c r="I5" s="21"/>
-      <c r="J5" s="22">
+      <c r="I5" s="20"/>
+      <c r="J5" s="21">
         <v>-2.2999999999999998</v>
       </c>
     </row>
@@ -6354,29 +5971,29 @@
       <c r="A6" t="s">
         <v>131</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="D6" s="24">
+      <c r="D6" s="23">
         <v>36.6</v>
       </c>
-      <c r="E6" s="24">
+      <c r="E6" s="23">
         <v>36.6</v>
       </c>
-      <c r="F6" s="24">
+      <c r="F6" s="23">
         <v>36.6</v>
       </c>
-      <c r="G6" s="24">
+      <c r="G6" s="23">
         <v>36.6</v>
       </c>
-      <c r="H6" s="24">
+      <c r="H6" s="23">
         <v>36.6</v>
       </c>
-      <c r="I6" s="24"/>
-      <c r="J6" s="25">
+      <c r="I6" s="23"/>
+      <c r="J6" s="24">
         <v>36.6</v>
       </c>
     </row>
@@ -6414,29 +6031,29 @@
       <c r="A8" t="s">
         <v>130</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="20" t="s">
         <v>133</v>
       </c>
-      <c r="D8" s="21">
+      <c r="D8" s="20">
         <v>42.6</v>
       </c>
-      <c r="E8" s="21">
+      <c r="E8" s="20">
         <v>41.5</v>
       </c>
-      <c r="F8" s="21">
+      <c r="F8" s="20">
         <v>38</v>
       </c>
-      <c r="G8" s="21">
+      <c r="G8" s="20">
         <v>34.5</v>
       </c>
-      <c r="H8" s="21">
+      <c r="H8" s="20">
         <v>30.6</v>
       </c>
-      <c r="I8" s="21"/>
-      <c r="J8" s="22">
+      <c r="I8" s="20"/>
+      <c r="J8" s="21">
         <v>23.7</v>
       </c>
     </row>
@@ -6497,13 +6114,292 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B17">
         <v>25</v>
       </c>
       <c r="C17">
         <f>30/(20+B17)</f>
         <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" t="s">
+        <v>148</v>
+      </c>
+      <c r="C20" t="s">
+        <v>149</v>
+      </c>
+      <c r="D20" t="s">
+        <v>150</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="G20" t="s">
+        <v>153</v>
+      </c>
+      <c r="H20" t="s">
+        <v>155</v>
+      </c>
+      <c r="I20" t="s">
+        <v>156</v>
+      </c>
+      <c r="J20" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A21" s="28">
+        <v>5</v>
+      </c>
+      <c r="B21" s="28" t="s">
+        <v>154</v>
+      </c>
+      <c r="C21" s="28">
+        <v>10</v>
+      </c>
+      <c r="D21" s="28">
+        <v>8</v>
+      </c>
+      <c r="E21" s="29">
+        <v>43.5</v>
+      </c>
+      <c r="F21" s="29">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="G21" s="28">
+        <v>0.88</v>
+      </c>
+      <c r="H21" s="28"/>
+      <c r="I21" s="28"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A22" s="28">
+        <v>5</v>
+      </c>
+      <c r="B22" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="C22" s="28">
+        <v>10</v>
+      </c>
+      <c r="D22" s="28">
+        <v>20</v>
+      </c>
+      <c r="E22" s="29">
+        <v>34.1</v>
+      </c>
+      <c r="F22" s="29">
+        <v>0.86</v>
+      </c>
+      <c r="G22" s="28">
+        <v>0.69</v>
+      </c>
+      <c r="H22" s="30">
+        <f>E21/E22</f>
+        <v>1.2756598240469208</v>
+      </c>
+      <c r="I22" s="30">
+        <f t="shared" ref="I22:J22" si="1">F21/F22</f>
+        <v>1.2674418604651163</v>
+      </c>
+      <c r="J22" s="10">
+        <f t="shared" si="1"/>
+        <v>1.2753623188405798</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>5</v>
+      </c>
+      <c r="B23" t="s">
+        <v>154</v>
+      </c>
+      <c r="C23">
+        <v>25</v>
+      </c>
+      <c r="D23">
+        <v>5.4</v>
+      </c>
+      <c r="E23" s="12">
+        <v>47.4</v>
+      </c>
+      <c r="F23" s="12">
+        <v>1.19</v>
+      </c>
+      <c r="G23">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>5</v>
+      </c>
+      <c r="B24" t="s">
+        <v>90</v>
+      </c>
+      <c r="C24">
+        <v>5</v>
+      </c>
+      <c r="D24">
+        <v>22.8</v>
+      </c>
+      <c r="E24" s="12">
+        <v>32.200000000000003</v>
+      </c>
+      <c r="F24" s="12">
+        <v>0.81</v>
+      </c>
+      <c r="G24">
+        <v>0.65</v>
+      </c>
+      <c r="H24" s="10">
+        <f>E23/E24</f>
+        <v>1.4720496894409936</v>
+      </c>
+      <c r="I24" s="10">
+        <f t="shared" ref="I24" si="2">F23/F24</f>
+        <v>1.4691358024691357</v>
+      </c>
+      <c r="J24" s="10">
+        <f t="shared" ref="J24" si="3">G23/G24</f>
+        <v>1.4769230769230768</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A25" s="28">
+        <v>6</v>
+      </c>
+      <c r="B25" s="28" t="s">
+        <v>154</v>
+      </c>
+      <c r="C25" s="28">
+        <v>10</v>
+      </c>
+      <c r="D25" s="28">
+        <v>27</v>
+      </c>
+      <c r="E25" s="29">
+        <v>26.5</v>
+      </c>
+      <c r="F25" s="29">
+        <v>1.19</v>
+      </c>
+      <c r="G25" s="28">
+        <v>1.03</v>
+      </c>
+      <c r="H25" s="30"/>
+      <c r="I25" s="30"/>
+      <c r="J25" s="10"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A26" s="28">
+        <v>6</v>
+      </c>
+      <c r="B26" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="C26" s="28">
+        <v>10</v>
+      </c>
+      <c r="D26" s="28">
+        <v>27</v>
+      </c>
+      <c r="E26" s="29">
+        <v>26.5</v>
+      </c>
+      <c r="F26" s="29">
+        <v>1.19</v>
+      </c>
+      <c r="G26" s="28">
+        <v>1.03</v>
+      </c>
+      <c r="H26" s="30">
+        <f>E25/E26</f>
+        <v>1</v>
+      </c>
+      <c r="I26" s="30">
+        <f t="shared" ref="I26" si="4">F25/F26</f>
+        <v>1</v>
+      </c>
+      <c r="J26" s="10"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>6</v>
+      </c>
+      <c r="B27" t="s">
+        <v>154</v>
+      </c>
+      <c r="C27">
+        <v>25</v>
+      </c>
+      <c r="D27">
+        <v>18.2</v>
+      </c>
+      <c r="E27" s="12">
+        <v>30.1</v>
+      </c>
+      <c r="F27" s="12">
+        <v>1.35</v>
+      </c>
+      <c r="G27" s="12">
+        <v>1.1599999999999999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>6</v>
+      </c>
+      <c r="B28" t="s">
+        <v>90</v>
+      </c>
+      <c r="C28">
+        <v>5</v>
+      </c>
+      <c r="D28">
+        <v>30.8</v>
+      </c>
+      <c r="E28" s="12">
+        <v>25.2</v>
+      </c>
+      <c r="F28" s="12">
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="G28" s="12">
+        <v>0.98</v>
+      </c>
+      <c r="H28" s="10">
+        <f>E27/E28</f>
+        <v>1.1944444444444446</v>
+      </c>
+      <c r="I28" s="10">
+        <f t="shared" ref="I28" si="5">F27/F28</f>
+        <v>1.1946902654867257</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="F29" s="12">
+        <f>F23-F24</f>
+        <v>0.37999999999999989</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="F30" s="12">
+        <f>F27-F28</f>
+        <v>0.2200000000000002</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -6512,7 +6408,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C2120DA-4889-CE46-967A-1E97B2CF047D}">
   <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -7076,7 +6972,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E4B153B-BE8A-8445-8BB9-AE4D4CAEE74C}">
   <dimension ref="A1:O88"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -11223,7 +11119,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55E721B4-ED8E-434B-9DEE-2C2B14F64426}">
   <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -12540,7 +12436,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BE2EFF2-13EC-F842-8DF0-C6F8E64FF8D5}">
   <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -12761,7 +12657,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7C0FFF9-DB26-954D-871D-A338BC7B0C37}">
   <dimension ref="A1:G122"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -15582,4 +15478,421 @@
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C764B46-5E34-3D45-A366-6036CFA976BB}">
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>478867</v>
+      </c>
+      <c r="C2">
+        <v>478992</v>
+      </c>
+      <c r="D2">
+        <v>478163</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>477459</v>
+      </c>
+      <c r="C3">
+        <v>478163</v>
+      </c>
+      <c r="D3">
+        <v>476688.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>475918</v>
+      </c>
+      <c r="C4">
+        <v>476688.5</v>
+      </c>
+      <c r="D4">
+        <v>475642.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>475367</v>
+      </c>
+      <c r="C5">
+        <v>475642.5</v>
+      </c>
+      <c r="D5">
+        <v>475200</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>475033</v>
+      </c>
+      <c r="C6">
+        <v>475200</v>
+      </c>
+      <c r="D6">
+        <v>474588.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>474144</v>
+      </c>
+      <c r="C7">
+        <v>474588.5</v>
+      </c>
+      <c r="D7">
+        <v>473750.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>473357</v>
+      </c>
+      <c r="C8">
+        <v>473750.5</v>
+      </c>
+      <c r="D8">
+        <v>473105.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>472854</v>
+      </c>
+      <c r="C9">
+        <v>473105.5</v>
+      </c>
+      <c r="D9">
+        <v>472383</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>471912</v>
+      </c>
+      <c r="C10">
+        <v>472383</v>
+      </c>
+      <c r="D10">
+        <v>471028</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>470144</v>
+      </c>
+      <c r="C11">
+        <v>471028</v>
+      </c>
+      <c r="D11">
+        <v>469836</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>469528</v>
+      </c>
+      <c r="C12">
+        <v>469836</v>
+      </c>
+      <c r="D12">
+        <v>469043.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>468559</v>
+      </c>
+      <c r="C13">
+        <v>469043.5</v>
+      </c>
+      <c r="D13">
+        <v>467805.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>467052</v>
+      </c>
+      <c r="C14">
+        <v>467805.5</v>
+      </c>
+      <c r="D14">
+        <v>466927</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A6B7A04-5F13-8A4E-9FE0-C5F28B59E7E3}">
+  <dimension ref="A1:P4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" t="s">
+        <v>8</v>
+      </c>
+      <c r="L1" t="s">
+        <v>86</v>
+      </c>
+      <c r="M1" t="s">
+        <v>85</v>
+      </c>
+      <c r="N1" t="s">
+        <v>84</v>
+      </c>
+      <c r="O1" t="s">
+        <v>89</v>
+      </c>
+      <c r="P1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A2" s="26">
+        <v>601</v>
+      </c>
+      <c r="B2" s="26">
+        <v>129045.2</v>
+      </c>
+      <c r="C2" s="26">
+        <v>474043.1</v>
+      </c>
+      <c r="D2" s="26">
+        <v>6</v>
+      </c>
+      <c r="E2" s="26">
+        <v>476.3</v>
+      </c>
+      <c r="F2" s="26">
+        <v>129515</v>
+      </c>
+      <c r="G2" s="26">
+        <v>473962</v>
+      </c>
+      <c r="H2" s="26">
+        <v>1</v>
+      </c>
+      <c r="I2" s="26">
+        <v>-2.6</v>
+      </c>
+      <c r="J2" s="26">
+        <v>-2.6</v>
+      </c>
+      <c r="K2" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="L2" s="26">
+        <v>0</v>
+      </c>
+      <c r="M2" s="26">
+        <v>-1.5580000000000001</v>
+      </c>
+      <c r="N2" s="26">
+        <v>-1.698</v>
+      </c>
+      <c r="O2" s="26">
+        <v>-1.5580000000000001</v>
+      </c>
+      <c r="P2" s="26">
+        <v>-1.698</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A3" s="26">
+        <v>602</v>
+      </c>
+      <c r="B3" s="26">
+        <v>129311.3</v>
+      </c>
+      <c r="C3" s="26">
+        <v>474110.7</v>
+      </c>
+      <c r="D3" s="26">
+        <v>6</v>
+      </c>
+      <c r="E3" s="26">
+        <v>225.7</v>
+      </c>
+      <c r="F3" s="26">
+        <v>129534</v>
+      </c>
+      <c r="G3" s="26">
+        <v>474072</v>
+      </c>
+      <c r="H3" s="26">
+        <v>1</v>
+      </c>
+      <c r="I3" s="26">
+        <v>-2.6</v>
+      </c>
+      <c r="J3" s="26">
+        <v>-2.6</v>
+      </c>
+      <c r="K3" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="L3" s="26">
+        <v>0</v>
+      </c>
+      <c r="M3" s="26">
+        <v>-1.415</v>
+      </c>
+      <c r="N3" s="26">
+        <v>-1.6359999999999999</v>
+      </c>
+      <c r="O3" s="26">
+        <v>-1.415</v>
+      </c>
+      <c r="P3" s="26">
+        <v>-1.6359999999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A4" s="26">
+        <v>603</v>
+      </c>
+      <c r="B4" s="26">
+        <v>129485.6</v>
+      </c>
+      <c r="C4" s="26">
+        <v>474227.9</v>
+      </c>
+      <c r="D4" s="26">
+        <v>6</v>
+      </c>
+      <c r="E4" s="26">
+        <v>73.900000000000006</v>
+      </c>
+      <c r="F4" s="26">
+        <v>129558</v>
+      </c>
+      <c r="G4" s="26">
+        <v>474215</v>
+      </c>
+      <c r="H4" s="26">
+        <v>1</v>
+      </c>
+      <c r="I4" s="26">
+        <v>-2.6</v>
+      </c>
+      <c r="J4" s="26">
+        <v>-2.6</v>
+      </c>
+      <c r="K4" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="L4" s="26">
+        <v>0</v>
+      </c>
+      <c r="M4" s="26">
+        <v>-1.196</v>
+      </c>
+      <c r="N4" s="26">
+        <v>-1.4850000000000001</v>
+      </c>
+      <c r="O4" s="26">
+        <v>-1.196</v>
+      </c>
+      <c r="P4" s="26">
+        <v>-1.4850000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Flow unde disk and strip added.
</commit_message>
<xml_diff>
--- a/Projects/ARK_RWS/images/peilbuizen/pb_tauw_XY.xlsx
+++ b/Projects/ARK_RWS/images/peilbuizen/pb_tauw_XY.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Theo/Development/python/mf6_tools/mf6lab/Projects/ARK_RWS/images/peilbuizen/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F148F20-8D91-4D40-BDF1-2E6726A06293}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66564BCF-1FEA-8A4E-ABF8-B74CBABE8A25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-1140" yWindow="-21520" windowWidth="32360" windowHeight="20720" activeTab="1" xr2:uid="{E4383F88-647D-C347-BE79-FF24D0CA7E92}"/>
+    <workbookView xWindow="-1140" yWindow="-21520" windowWidth="32360" windowHeight="20720" activeTab="2" xr2:uid="{E4383F88-647D-C347-BE79-FF24D0CA7E92}"/>
   </bookViews>
   <sheets>
     <sheet name="pbTauw" sheetId="1" r:id="rId1"/>
@@ -270,7 +270,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="160">
   <si>
     <t>x</t>
   </si>
@@ -315,9 +315,6 @@
   </si>
   <si>
     <t>E</t>
-  </si>
-  <si>
-    <t>onzeker_bk_laag</t>
   </si>
   <si>
     <t>inkanaal</t>
@@ -745,6 +742,15 @@
   <si>
     <t>ARK temp (2024, 2025)</t>
   </si>
+  <si>
+    <t>h(01-02-26)</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>naam</t>
+  </si>
 </sst>
 </file>
 
@@ -948,7 +954,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -988,6 +994,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1015,8 +1024,8 @@
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>533400</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
       <xdr:row>45</xdr:row>
       <xdr:rowOff>32327</xdr:rowOff>
     </xdr:to>
@@ -1534,19 +1543,19 @@
         <v>8</v>
       </c>
       <c r="L1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="M1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="N1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O1" t="s">
+        <v>88</v>
+      </c>
+      <c r="P1" t="s">
         <v>89</v>
-      </c>
-      <c r="P1" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
@@ -5670,33 +5679,33 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E1" t="s">
+        <v>118</v>
+      </c>
+      <c r="F1" t="s">
+        <v>123</v>
+      </c>
+      <c r="G1" t="s">
+        <v>122</v>
+      </c>
+      <c r="H1" t="s">
         <v>121</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="D1" t="s">
-        <v>120</v>
-      </c>
-      <c r="E1" t="s">
-        <v>119</v>
-      </c>
-      <c r="F1" t="s">
-        <v>124</v>
-      </c>
-      <c r="G1" t="s">
-        <v>123</v>
-      </c>
-      <c r="H1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>5</v>
@@ -5723,7 +5732,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>14</v>
@@ -5751,7 +5760,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>5</v>
@@ -5779,7 +5788,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>14</v>
@@ -5824,42 +5833,42 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B1" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="D1" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="C1" s="13" t="s">
-        <v>135</v>
-      </c>
-      <c r="D1" s="14" t="s">
+      <c r="E1" s="14" t="s">
         <v>137</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="F1" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="G1" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="H1" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="I1" s="14" t="s">
         <v>141</v>
       </c>
-      <c r="I1" s="14" t="s">
-        <v>142</v>
-      </c>
       <c r="J1" s="14" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D2" s="23">
         <v>1E-3</v>
@@ -5885,10 +5894,10 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B3" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D3" s="16">
         <v>-0.4</v>
@@ -5912,13 +5921,13 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D4" s="11">
         <v>-0.65500000000000003</v>
@@ -5942,10 +5951,10 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B5" s="19" t="s">
+        <v>142</v>
+      </c>
+      <c r="C5" s="20" t="s">
         <v>143</v>
-      </c>
-      <c r="C5" s="20" t="s">
-        <v>144</v>
       </c>
       <c r="D5" s="20">
         <v>-2.2999999999999998</v>
@@ -5969,13 +5978,13 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D6" s="23">
         <v>36.6</v>
@@ -5999,13 +6008,13 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D7" s="16">
         <v>10.8</v>
@@ -6029,13 +6038,13 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B8" s="19" t="s">
         <v>130</v>
       </c>
-      <c r="B8" s="19" t="s">
-        <v>131</v>
-      </c>
       <c r="C8" s="20" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D8" s="20">
         <v>42.6</v>
@@ -6059,7 +6068,7 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D10" s="11">
         <f>D4-$J$4</f>
@@ -6128,31 +6137,31 @@
         <v>9</v>
       </c>
       <c r="B20" t="s">
+        <v>147</v>
+      </c>
+      <c r="C20" t="s">
         <v>148</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>149</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="E20" s="12" t="s">
+      <c r="F20" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="F20" s="12" t="s">
+      <c r="G20" t="s">
         <v>152</v>
       </c>
-      <c r="G20" t="s">
-        <v>153</v>
-      </c>
       <c r="H20" t="s">
+        <v>154</v>
+      </c>
+      <c r="I20" t="s">
         <v>155</v>
       </c>
-      <c r="I20" t="s">
-        <v>156</v>
-      </c>
       <c r="J20" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
@@ -6160,7 +6169,7 @@
         <v>5</v>
       </c>
       <c r="B21" s="28" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C21" s="28">
         <v>10</v>
@@ -6185,7 +6194,7 @@
         <v>5</v>
       </c>
       <c r="B22" s="28" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C22" s="28">
         <v>10</v>
@@ -6220,7 +6229,7 @@
         <v>5</v>
       </c>
       <c r="B23" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C23">
         <v>25</v>
@@ -6243,7 +6252,7 @@
         <v>5</v>
       </c>
       <c r="B24" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C24">
         <v>5</v>
@@ -6278,7 +6287,7 @@
         <v>6</v>
       </c>
       <c r="B25" s="28" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C25" s="28">
         <v>10</v>
@@ -6304,7 +6313,7 @@
         <v>6</v>
       </c>
       <c r="B26" s="28" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C26" s="28">
         <v>10</v>
@@ -6336,7 +6345,7 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C27">
         <v>25</v>
@@ -6359,7 +6368,7 @@
         <v>6</v>
       </c>
       <c r="B28" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C28">
         <v>5</v>
@@ -6399,7 +6408,7 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -6410,56 +6419,67 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C2120DA-4889-CE46-967A-1E97B2CF047D}">
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="5.83203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.83203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B1" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="E1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="E1" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="K1" t="s">
-        <v>15</v>
-      </c>
-      <c r="L1" t="s">
+      <c r="K1" s="12"/>
+      <c r="L1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="N1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>1</v>
+      <c r="N1" s="12" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="B2" s="3">
         <v>129709.5</v>
@@ -6471,7 +6491,7 @@
         <v>4</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F2" t="s">
         <v>5</v>
@@ -6489,9 +6509,6 @@
         <f t="shared" ref="J2:J5" si="0">H2-I2</f>
         <v>2.5</v>
       </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
       <c r="L2">
         <v>-0.4</v>
       </c>
@@ -6499,13 +6516,16 @@
         <v>-0.4</v>
       </c>
       <c r="N2">
-        <f t="shared" ref="N2:N11" si="1">VLOOKUP("Pb"&amp;$A2,yyy,7,FALSE)</f>
+        <f>VLOOKUP("Pb"&amp;$O2,yyy,7,FALSE)</f>
         <v>-1.3220000000000001</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>2</v>
+      <c r="O2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="B3" s="3">
         <v>129824.5</v>
@@ -6517,7 +6537,7 @@
         <v>4</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F3" t="s">
         <v>14</v>
@@ -6535,9 +6555,6 @@
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
       <c r="L3">
         <v>-2.2999999999999998</v>
       </c>
@@ -6545,13 +6562,16 @@
         <v>-2.2999999999999998</v>
       </c>
       <c r="N3">
-        <f t="shared" si="1"/>
+        <f>VLOOKUP("Pb"&amp;$O3,yyy,7,FALSE)</f>
         <v>-1.3759999999999999</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>3</v>
+      <c r="O3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>20</v>
       </c>
       <c r="B4" s="3">
         <v>129798.5</v>
@@ -6563,7 +6583,7 @@
         <v>4</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F4" t="s">
         <v>14</v>
@@ -6581,8 +6601,8 @@
         <f t="shared" si="0"/>
         <v>3.25</v>
       </c>
-      <c r="K4">
-        <v>1</v>
+      <c r="K4" t="s">
+        <v>158</v>
       </c>
       <c r="L4">
         <v>-0.4</v>
@@ -6591,13 +6611,16 @@
         <v>-0.4</v>
       </c>
       <c r="N4">
-        <f t="shared" si="1"/>
+        <f>VLOOKUP("Pb"&amp;$O4,yyy,7,FALSE)</f>
         <v>-1.1439999999999999</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>4</v>
+      <c r="O4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="B5" s="3">
         <v>129629.5</v>
@@ -6609,7 +6632,7 @@
         <v>5</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F5" t="s">
         <v>5</v>
@@ -6627,9 +6650,6 @@
         <f t="shared" si="0"/>
         <v>1.75</v>
       </c>
-      <c r="K5">
-        <v>0</v>
-      </c>
       <c r="L5">
         <v>-0.4</v>
       </c>
@@ -6637,13 +6657,16 @@
         <v>-0.4</v>
       </c>
       <c r="N5">
-        <f t="shared" si="1"/>
+        <f>VLOOKUP("Pb"&amp;$O5,yyy,7,FALSE)</f>
         <v>-1.403</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>5</v>
+      <c r="O5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="B6" s="3">
         <v>129720.5</v>
@@ -6655,7 +6678,7 @@
         <v>5</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F6" t="s">
         <v>14</v>
@@ -6673,9 +6696,6 @@
         <f>H6-I6</f>
         <v>0.75</v>
       </c>
-      <c r="K6">
-        <v>0</v>
-      </c>
       <c r="L6">
         <v>-0.4</v>
       </c>
@@ -6683,13 +6703,16 @@
         <v>-0.4</v>
       </c>
       <c r="N6">
-        <f t="shared" si="1"/>
+        <f>VLOOKUP("Pb"&amp;$O6,yyy,7,FALSE)</f>
         <v>-1.3819999999999999</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>6</v>
+      <c r="O6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="B7" s="3">
         <v>129720.5</v>
@@ -6701,7 +6724,7 @@
         <v>5</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F7" t="s">
         <v>14</v>
@@ -6716,11 +6739,11 @@
         <v>-4.25</v>
       </c>
       <c r="J7">
-        <f t="shared" ref="J7:J11" si="2">H7-I7</f>
+        <f t="shared" ref="J7:J11" si="1">H7-I7</f>
         <v>2.75</v>
       </c>
-      <c r="K7">
-        <v>1</v>
+      <c r="K7" t="s">
+        <v>158</v>
       </c>
       <c r="L7">
         <v>-2.2999999999999998</v>
@@ -6729,13 +6752,16 @@
         <v>-2.2999999999999998</v>
       </c>
       <c r="N7">
-        <f t="shared" si="1"/>
+        <f>VLOOKUP("Pb"&amp;$O7,yyy,7,FALSE)</f>
         <v>-1.502</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>7</v>
+      <c r="O7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>24</v>
       </c>
       <c r="B8" s="3">
         <v>129129.5</v>
@@ -6747,7 +6773,7 @@
         <v>9</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F8" t="s">
         <v>5</v>
@@ -6762,11 +6788,8 @@
         <v>-6.75</v>
       </c>
       <c r="J8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>3</v>
-      </c>
-      <c r="K8">
-        <v>0</v>
       </c>
       <c r="L8">
         <v>-0.4</v>
@@ -6775,13 +6798,16 @@
         <v>-0.4</v>
       </c>
       <c r="N8">
-        <f t="shared" si="1"/>
+        <f>VLOOKUP("Pb"&amp;$O8,yyy,7,FALSE)</f>
         <v>-1.4890000000000001</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>8</v>
+      <c r="O8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="B9" s="3">
         <v>129212.5</v>
@@ -6793,7 +6819,7 @@
         <v>9</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F9" t="s">
         <v>14</v>
@@ -6808,11 +6834,8 @@
         <v>-7.25</v>
       </c>
       <c r="J9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>3.25</v>
-      </c>
-      <c r="K9">
-        <v>0</v>
       </c>
       <c r="L9">
         <v>-2.25</v>
@@ -6821,13 +6844,16 @@
         <v>-2.25</v>
       </c>
       <c r="N9">
-        <f t="shared" si="1"/>
+        <f>VLOOKUP("Pb"&amp;$O9,yyy,7,FALSE)</f>
         <v>-1.5649999999999999</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>9</v>
+      <c r="O9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>26</v>
       </c>
       <c r="B10" s="3">
         <v>129244.5</v>
@@ -6839,7 +6865,7 @@
         <v>9</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F10" t="s">
         <v>14</v>
@@ -6854,11 +6880,11 @@
         <v>-7.25</v>
       </c>
       <c r="J10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.25</v>
       </c>
-      <c r="K10">
-        <v>1</v>
+      <c r="K10" t="s">
+        <v>158</v>
       </c>
       <c r="L10">
         <v>-0.4</v>
@@ -6867,13 +6893,16 @@
         <v>-0.4</v>
       </c>
       <c r="N10">
-        <f t="shared" si="1"/>
+        <f>VLOOKUP("Pb"&amp;$O10,yyy,7,FALSE)</f>
         <v>-1.4810000000000001</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>10</v>
+      <c r="O10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>86</v>
       </c>
       <c r="B11" s="3">
         <v>128657.5</v>
@@ -6885,7 +6914,7 @@
         <v>11</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F11" t="s">
         <v>5</v>
@@ -6900,11 +6929,8 @@
         <v>-7.25</v>
       </c>
       <c r="J11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>4.5</v>
-      </c>
-      <c r="K11">
-        <v>0</v>
       </c>
       <c r="L11">
         <v>-0.4</v>
@@ -6913,19 +6939,22 @@
         <v>-0.4</v>
       </c>
       <c r="N11">
-        <f t="shared" si="1"/>
+        <f>VLOOKUP("Pb"&amp;$O11,yyy,7,FALSE)</f>
         <v>-1.5589999999999999</v>
       </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
     </row>
@@ -7009,19 +7038,19 @@
         <v>7</v>
       </c>
       <c r="K1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="L1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N1" t="s">
+        <v>88</v>
+      </c>
+      <c r="O1" t="s">
         <v>89</v>
-      </c>
-      <c r="O1" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
@@ -11126,7 +11155,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B1" s="2">
         <v>45682</v>
@@ -11143,7 +11172,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B2" s="2">
         <v>45682</v>
@@ -11160,7 +11189,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B3" s="2">
         <v>45682</v>
@@ -11177,7 +11206,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B4" s="2">
         <v>45682</v>
@@ -11194,7 +11223,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B5" s="2">
         <v>45682</v>
@@ -11211,7 +11240,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B6" s="2">
         <v>45682</v>
@@ -11228,7 +11257,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B7" s="2">
         <v>45682</v>
@@ -11245,7 +11274,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B8" s="2">
         <v>45682</v>
@@ -11262,7 +11291,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B9" s="2">
         <v>45682</v>
@@ -11279,7 +11308,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B10" s="2">
         <v>45682</v>
@@ -11296,7 +11325,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B11" s="2">
         <v>45682</v>
@@ -11316,7 +11345,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B12" s="2">
         <v>45682</v>
@@ -11336,7 +11365,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B13" s="2">
         <v>45682</v>
@@ -11356,7 +11385,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B14" s="2">
         <v>45682</v>
@@ -11376,7 +11405,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B15" s="2">
         <v>45682</v>
@@ -11393,7 +11422,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B16" s="2">
         <v>45682</v>
@@ -11413,7 +11442,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B17" s="2">
         <v>45682</v>
@@ -11430,7 +11459,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B18" s="2">
         <v>45682</v>
@@ -11447,7 +11476,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B19" s="2">
         <v>45682</v>
@@ -11461,7 +11490,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B20" s="2">
         <v>45682</v>
@@ -11481,7 +11510,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B21" s="2">
         <v>45682</v>
@@ -11504,7 +11533,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B22" s="2">
         <v>45682</v>
@@ -11527,7 +11556,7 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B23" s="2">
         <v>45682</v>
@@ -11550,7 +11579,7 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B24" s="2">
         <v>45682</v>
@@ -11573,7 +11602,7 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B25" s="2">
         <v>45682</v>
@@ -11596,7 +11625,7 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B26" s="2">
         <v>45682</v>
@@ -11613,7 +11642,7 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B27" s="2">
         <v>45682</v>
@@ -11636,7 +11665,7 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B28" s="2">
         <v>45682</v>
@@ -11656,7 +11685,7 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B29" s="2">
         <v>45682</v>
@@ -11679,7 +11708,7 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B30" s="2">
         <v>45682</v>
@@ -11696,7 +11725,7 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B31" s="2">
         <v>45682</v>
@@ -11719,7 +11748,7 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B32" s="2">
         <v>45682</v>
@@ -11742,7 +11771,7 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B33" s="2">
         <v>45682</v>
@@ -11762,7 +11791,7 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B34" s="2">
         <v>45682</v>
@@ -11782,7 +11811,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B35" s="2">
         <v>45682</v>
@@ -11802,7 +11831,7 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B36" s="2">
         <v>45682</v>
@@ -11822,7 +11851,7 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B37" s="2">
         <v>45682</v>
@@ -11839,7 +11868,7 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B38" s="2">
         <v>45682</v>
@@ -11859,7 +11888,7 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B39" s="2">
         <v>45682</v>
@@ -11879,7 +11908,7 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B40" s="2">
         <v>45682</v>
@@ -11896,7 +11925,7 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B41" s="2">
         <v>45682</v>
@@ -11916,7 +11945,7 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B42" s="2">
         <v>45682</v>
@@ -11936,7 +11965,7 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B43" s="2">
         <v>45682</v>
@@ -11953,7 +11982,7 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B44" s="2">
         <v>45682</v>
@@ -11973,7 +12002,7 @@
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B45" s="2">
         <v>45682</v>
@@ -11993,7 +12022,7 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B46" s="2">
         <v>45682</v>
@@ -12013,7 +12042,7 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B47" s="2">
         <v>45682</v>
@@ -12033,7 +12062,7 @@
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B48" s="2">
         <v>45682</v>
@@ -12053,7 +12082,7 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B49" s="2">
         <v>45682</v>
@@ -12073,7 +12102,7 @@
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B50" s="2">
         <v>45682</v>
@@ -12093,7 +12122,7 @@
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B51" s="2">
         <v>45682</v>
@@ -12113,7 +12142,7 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B52" s="2">
         <v>45682</v>
@@ -12133,7 +12162,7 @@
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B53" s="2">
         <v>45682</v>
@@ -12153,7 +12182,7 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B54" s="2">
         <v>45682</v>
@@ -12176,7 +12205,7 @@
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B55" s="2">
         <v>45682</v>
@@ -12199,7 +12228,7 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B56" s="2">
         <v>45682</v>
@@ -12222,7 +12251,7 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B57" s="2">
         <v>45682</v>
@@ -12245,7 +12274,7 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B58" s="2">
         <v>45682</v>
@@ -12265,7 +12294,7 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B59" s="2">
         <v>45682</v>
@@ -12285,7 +12314,7 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B60" s="2">
         <v>45682</v>
@@ -12302,7 +12331,7 @@
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B61" s="2">
         <v>45682</v>
@@ -12319,7 +12348,7 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B62" s="2">
         <v>45682</v>
@@ -12339,7 +12368,7 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B63" s="2">
         <v>45682</v>
@@ -12356,7 +12385,7 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B64" s="2">
         <v>45682</v>
@@ -12376,7 +12405,7 @@
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B65" s="2">
         <v>45682</v>
@@ -12396,7 +12425,7 @@
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B66" s="2">
         <v>45682</v>
@@ -12416,7 +12445,7 @@
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B67" s="2">
         <v>45682</v>
@@ -12443,34 +12472,34 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="B1" t="s">
-        <v>92</v>
-      </c>
       <c r="C1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1" t="s">
         <v>98</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>99</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>113</v>
+      </c>
+      <c r="G1" t="s">
         <v>100</v>
       </c>
-      <c r="F1" t="s">
-        <v>114</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
+        <v>96</v>
+      </c>
+      <c r="I1" t="s">
         <v>101</v>
       </c>
-      <c r="H1" t="s">
-        <v>97</v>
-      </c>
-      <c r="I1" t="s">
-        <v>102</v>
-      </c>
       <c r="J1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
@@ -12500,13 +12529,13 @@
         <v>200</v>
       </c>
       <c r="H2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
@@ -12536,13 +12565,13 @@
         <v>800</v>
       </c>
       <c r="H3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="J3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
@@ -12572,13 +12601,13 @@
         <v>28</v>
       </c>
       <c r="H4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
@@ -12608,13 +12637,13 @@
         <v>25</v>
       </c>
       <c r="H5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
@@ -12643,13 +12672,13 @@
         <v>9.5</v>
       </c>
       <c r="H6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -12667,7 +12696,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>0</v>
@@ -15490,13 +15519,13 @@
         <v>9</v>
       </c>
       <c r="B1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C1" t="s">
         <v>115</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>116</v>
-      </c>
-      <c r="D1" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -15726,19 +15755,19 @@
         <v>8</v>
       </c>
       <c r="L1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="M1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="N1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O1" t="s">
+        <v>88</v>
+      </c>
+      <c r="P1" t="s">
         <v>89</v>
-      </c>
-      <c r="P1" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Reporting with some improvements of the model. Underwater bench added, sheet-piling resistance adapted.
</commit_message>
<xml_diff>
--- a/Projects/ARK_RWS/images/peilbuizen/pb_tauw_XY.xlsx
+++ b/Projects/ARK_RWS/images/peilbuizen/pb_tauw_XY.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Theo/Development/python/mf6_tools/mf6lab/Projects/ARK_RWS/images/peilbuizen/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66564BCF-1FEA-8A4E-ABF8-B74CBABE8A25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{188BE82C-16D4-F249-B3CE-6BBC21F3961D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-1140" yWindow="-21520" windowWidth="32360" windowHeight="20720" activeTab="2" xr2:uid="{E4383F88-647D-C347-BE79-FF24D0CA7E92}"/>
   </bookViews>
@@ -270,7 +270,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="159">
   <si>
     <t>x</t>
   </si>
@@ -747,9 +747,6 @@
   </si>
   <si>
     <t>?</t>
-  </si>
-  <si>
-    <t>naam</t>
   </si>
 </sst>
 </file>
@@ -6437,7 +6434,7 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>159</v>
+        <v>2</v>
       </c>
       <c r="B1" s="31" t="s">
         <v>0</v>
@@ -6478,8 +6475,8 @@
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>18</v>
+      <c r="A2" s="1">
+        <v>1</v>
       </c>
       <c r="B2" s="3">
         <v>129709.5</v>
@@ -6516,7 +6513,7 @@
         <v>-0.4</v>
       </c>
       <c r="N2">
-        <f>VLOOKUP("Pb"&amp;$O2,yyy,7,FALSE)</f>
+        <f t="shared" ref="N2:N11" si="1">VLOOKUP("Pb"&amp;$O2,yyy,7,FALSE)</f>
         <v>-1.3220000000000001</v>
       </c>
       <c r="O2">
@@ -6524,8 +6521,8 @@
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>19</v>
+      <c r="A3" s="1">
+        <v>2</v>
       </c>
       <c r="B3" s="3">
         <v>129824.5</v>
@@ -6562,7 +6559,7 @@
         <v>-2.2999999999999998</v>
       </c>
       <c r="N3">
-        <f>VLOOKUP("Pb"&amp;$O3,yyy,7,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>-1.3759999999999999</v>
       </c>
       <c r="O3">
@@ -6570,8 +6567,8 @@
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>20</v>
+      <c r="A4" s="1">
+        <v>3</v>
       </c>
       <c r="B4" s="3">
         <v>129798.5</v>
@@ -6611,7 +6608,7 @@
         <v>-0.4</v>
       </c>
       <c r="N4">
-        <f>VLOOKUP("Pb"&amp;$O4,yyy,7,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>-1.1439999999999999</v>
       </c>
       <c r="O4">
@@ -6619,8 +6616,8 @@
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>21</v>
+      <c r="A5" s="1">
+        <v>4</v>
       </c>
       <c r="B5" s="3">
         <v>129629.5</v>
@@ -6657,7 +6654,7 @@
         <v>-0.4</v>
       </c>
       <c r="N5">
-        <f>VLOOKUP("Pb"&amp;$O5,yyy,7,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>-1.403</v>
       </c>
       <c r="O5">
@@ -6665,8 +6662,8 @@
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>22</v>
+      <c r="A6" s="1">
+        <v>5</v>
       </c>
       <c r="B6" s="3">
         <v>129720.5</v>
@@ -6703,7 +6700,7 @@
         <v>-0.4</v>
       </c>
       <c r="N6">
-        <f>VLOOKUP("Pb"&amp;$O6,yyy,7,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>-1.3819999999999999</v>
       </c>
       <c r="O6">
@@ -6711,8 +6708,8 @@
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>23</v>
+      <c r="A7" s="1">
+        <v>6</v>
       </c>
       <c r="B7" s="3">
         <v>129720.5</v>
@@ -6739,7 +6736,7 @@
         <v>-4.25</v>
       </c>
       <c r="J7">
-        <f t="shared" ref="J7:J11" si="1">H7-I7</f>
+        <f t="shared" ref="J7:J11" si="2">H7-I7</f>
         <v>2.75</v>
       </c>
       <c r="K7" t="s">
@@ -6752,7 +6749,7 @@
         <v>-2.2999999999999998</v>
       </c>
       <c r="N7">
-        <f>VLOOKUP("Pb"&amp;$O7,yyy,7,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>-1.502</v>
       </c>
       <c r="O7">
@@ -6760,8 +6757,8 @@
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
-        <v>24</v>
+      <c r="A8" s="1">
+        <v>7</v>
       </c>
       <c r="B8" s="3">
         <v>129129.5</v>
@@ -6788,7 +6785,7 @@
         <v>-6.75</v>
       </c>
       <c r="J8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="L8">
@@ -6798,7 +6795,7 @@
         <v>-0.4</v>
       </c>
       <c r="N8">
-        <f>VLOOKUP("Pb"&amp;$O8,yyy,7,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>-1.4890000000000001</v>
       </c>
       <c r="O8">
@@ -6806,8 +6803,8 @@
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>25</v>
+      <c r="A9" s="1">
+        <v>8</v>
       </c>
       <c r="B9" s="3">
         <v>129212.5</v>
@@ -6834,7 +6831,7 @@
         <v>-7.25</v>
       </c>
       <c r="J9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.25</v>
       </c>
       <c r="L9">
@@ -6844,7 +6841,7 @@
         <v>-2.25</v>
       </c>
       <c r="N9">
-        <f>VLOOKUP("Pb"&amp;$O9,yyy,7,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>-1.5649999999999999</v>
       </c>
       <c r="O9">
@@ -6852,8 +6849,8 @@
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>26</v>
+      <c r="A10" s="1">
+        <v>9</v>
       </c>
       <c r="B10" s="3">
         <v>129244.5</v>
@@ -6880,7 +6877,7 @@
         <v>-7.25</v>
       </c>
       <c r="J10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4.25</v>
       </c>
       <c r="K10" t="s">
@@ -6893,7 +6890,7 @@
         <v>-0.4</v>
       </c>
       <c r="N10">
-        <f>VLOOKUP("Pb"&amp;$O10,yyy,7,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>-1.4810000000000001</v>
       </c>
       <c r="O10">
@@ -6901,8 +6898,8 @@
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
-        <v>86</v>
+      <c r="A11" s="1">
+        <v>10</v>
       </c>
       <c r="B11" s="3">
         <v>128657.5</v>
@@ -6929,7 +6926,7 @@
         <v>-7.25</v>
       </c>
       <c r="J11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4.5</v>
       </c>
       <c r="L11">
@@ -6939,7 +6936,7 @@
         <v>-0.4</v>
       </c>
       <c r="N11">
-        <f>VLOOKUP("Pb"&amp;$O11,yyy,7,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>-1.5589999999999999</v>
       </c>
       <c r="O11">

</xml_diff>